<commit_message>
Atualiza├º├úo autom├ítica (24/02/2026  8:15:08,23)
</commit_message>
<xml_diff>
--- a/rejeito.xlsx
+++ b/rejeito.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PLANILHAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{30422DC8-83FF-4DC4-8E32-5425E0346A44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{798F27DA-7352-4B62-8567-053B09BACDB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3585" yWindow="3585" windowWidth="21600" windowHeight="11295" xr2:uid="{11873F4D-6B6C-473D-B515-5F114D05EC28}"/>
+    <workbookView xWindow="3585" yWindow="3585" windowWidth="21600" windowHeight="11295" xr2:uid="{07B4FCB3-FF16-4E63-8B27-07285E70AFC4}"/>
   </bookViews>
   <sheets>
     <sheet name="rejeito" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="113">
   <si>
     <t>Dados</t>
   </si>
@@ -140,6 +140,9 @@
   </si>
   <si>
     <t>18/02/2026</t>
+  </si>
+  <si>
+    <t>23/02/2026</t>
   </si>
   <si>
     <t>02/01/2026</t>
@@ -900,8 +903,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26AF294C-3261-4767-A4BB-7A022C8C8839}">
-  <dimension ref="A1:O80"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3CA8AB7-A591-4CD1-85BC-46C85D7EFCC6}">
+  <dimension ref="A1:O82"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.42578125" customWidth="1"/>
@@ -932,14 +935,14 @@
       <c r="F1" s="11"/>
       <c r="G1" s="11"/>
       <c r="H1" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="I1" s="11"/>
       <c r="J1" s="11"/>
       <c r="K1" s="11"/>
       <c r="L1" s="11"/>
       <c r="M1" s="11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="N1" s="11"/>
       <c r="O1" s="11"/>
@@ -953,40 +956,40 @@
         <v>9</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" spans="1:15" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1025,25 +1028,25 @@
         <v>46046.443344907406</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I4" s="7">
         <v>1406207</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M4" s="10"/>
       <c r="N4" s="10">
@@ -1066,25 +1069,25 @@
         <v>46046.553217592591</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I5" s="7">
         <v>1406207</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M5" s="10"/>
       <c r="N5" s="10">
@@ -1107,25 +1110,25 @@
         <v>46050.493333333332</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I6" s="7">
         <v>1411349</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L6" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M6" s="10"/>
       <c r="N6" s="10">
@@ -1148,25 +1151,25 @@
         <v>46051.555428240739</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I7" s="7">
         <v>1411348</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="M7" s="10"/>
       <c r="N7" s="10">
@@ -1189,25 +1192,25 @@
         <v>46053.377129629633</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I8" s="7">
         <v>1409954</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M8" s="10"/>
       <c r="N8" s="10">
@@ -1230,25 +1233,25 @@
         <v>46062.302418981482</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I9" s="7">
         <v>1411984</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L9" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="M9" s="10"/>
       <c r="N9" s="10">
@@ -1271,25 +1274,25 @@
         <v>46062.570879629631</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I10" s="7">
         <v>1411984</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="M10" s="10"/>
       <c r="N10" s="10">
@@ -1312,25 +1315,25 @@
         <v>46064.297777777778</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I11" s="7">
         <v>1411984</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L11" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="M11" s="10"/>
       <c r="N11" s="10">
@@ -1353,25 +1356,25 @@
         <v>46064.455104166664</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I12" s="7">
         <v>1411990</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M12" s="10"/>
       <c r="N12" s="10">
@@ -1394,25 +1397,25 @@
         <v>46028.331469907411</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I13" s="7">
         <v>1402958</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L13" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M13" s="10"/>
       <c r="N13" s="10">
@@ -1435,25 +1438,25 @@
         <v>46030.306192129632</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I14" s="7">
         <v>1394721</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L14" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M14" s="10"/>
       <c r="N14" s="10">
@@ -1476,25 +1479,25 @@
         <v>46031.443101851852</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I15" s="7">
         <v>1394721</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M15" s="10"/>
       <c r="N15" s="10">
@@ -1517,25 +1520,25 @@
         <v>46035.530381944445</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I16" s="7">
         <v>1394721</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L16" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M16" s="10"/>
       <c r="N16" s="10">
@@ -1558,25 +1561,25 @@
         <v>46046.391701388886</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I17" s="7">
         <v>1410340</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L17" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M17" s="10"/>
       <c r="N17" s="10">
@@ -1599,25 +1602,25 @@
         <v>46046.516597222224</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I18" s="7">
         <v>1410340</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L18" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M18" s="10"/>
       <c r="N18" s="10">
@@ -1640,25 +1643,25 @@
         <v>46048.278912037036</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I19" s="7">
         <v>1410340</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K19" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L19" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M19" s="10"/>
       <c r="N19" s="10">
@@ -1681,25 +1684,25 @@
         <v>46051.403391203705</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I20" s="7">
         <v>1410340</v>
       </c>
       <c r="J20" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K20" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L20" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M20" s="10"/>
       <c r="N20" s="10">
@@ -1722,25 +1725,25 @@
         <v>46053.550381944442</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I21" s="7">
         <v>1411706</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L21" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="M21" s="10"/>
       <c r="N21" s="10">
@@ -1763,25 +1766,25 @@
         <v>46057.413171296299</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I22" s="7">
         <v>1411704</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L22" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M22" s="10"/>
       <c r="N22" s="10">
@@ -1804,25 +1807,25 @@
         <v>46058.357476851852</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I23" s="7">
         <v>1411704</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L23" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M23" s="10"/>
       <c r="N23" s="10">
@@ -1845,25 +1848,25 @@
         <v>46058.531793981485</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I24" s="7">
         <v>1411704</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L24" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M24" s="10"/>
       <c r="N24" s="10">
@@ -1886,25 +1889,25 @@
         <v>46067.433020833334</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I25" s="7">
         <v>1418256</v>
       </c>
       <c r="J25" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L25" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M25" s="10"/>
       <c r="N25" s="10">
@@ -1927,25 +1930,25 @@
         <v>46073.579664351855</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I26" s="7">
         <v>1422511</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L26" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M26" s="10"/>
       <c r="N26" s="10">
@@ -1968,25 +1971,25 @@
         <v>46027.4840625</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I27" s="7">
         <v>1404289</v>
       </c>
       <c r="J27" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L27" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M27" s="10"/>
       <c r="N27" s="10">
@@ -2009,25 +2012,25 @@
         <v>46030.397997685184</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I28" s="7">
         <v>1394724</v>
       </c>
       <c r="J28" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L28" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M28" s="10"/>
       <c r="N28" s="10">
@@ -2050,25 +2053,25 @@
         <v>46030.408148148148</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I29" s="7">
         <v>1394724</v>
       </c>
       <c r="J29" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L29" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M29" s="10"/>
       <c r="N29" s="10">
@@ -2091,25 +2094,25 @@
         <v>46030.478854166664</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G30" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I30" s="7">
         <v>1394724</v>
       </c>
       <c r="J30" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L30" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M30" s="10"/>
       <c r="N30" s="10">
@@ -2132,25 +2135,25 @@
         <v>46030.561284722222</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G31" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I31" s="7">
         <v>1394724</v>
       </c>
       <c r="J31" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L31" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M31" s="10"/>
       <c r="N31" s="10">
@@ -2173,25 +2176,25 @@
         <v>46035.478368055556</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G32" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I32" s="7">
         <v>1394724</v>
       </c>
       <c r="J32" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L32" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M32" s="10"/>
       <c r="N32" s="10">
@@ -2214,25 +2217,25 @@
         <v>46043.385474537034</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G33" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I33" s="7">
         <v>1394724</v>
       </c>
       <c r="J33" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L33" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M33" s="10"/>
       <c r="N33" s="10">
@@ -2255,25 +2258,25 @@
         <v>46043.565196759257</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G34" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I34" s="7">
         <v>1394724</v>
       </c>
       <c r="J34" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L34" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M34" s="10"/>
       <c r="N34" s="10">
@@ -2296,25 +2299,25 @@
         <v>46069.559953703705</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G35" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I35" s="7">
         <v>1421099</v>
       </c>
       <c r="J35" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K35" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L35" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M35" s="10"/>
       <c r="N35" s="10">
@@ -2337,25 +2340,25 @@
         <v>46035.47824074074</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G36" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H36" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I36" s="7">
         <v>1404958</v>
       </c>
       <c r="J36" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L36" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M36" s="10"/>
       <c r="N36" s="10">
@@ -2378,25 +2381,25 @@
         <v>46043.385196759256</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G37" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H37" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I37" s="7">
         <v>1405794</v>
       </c>
       <c r="J37" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L37" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M37" s="10"/>
       <c r="N37" s="10">
@@ -2419,25 +2422,25 @@
         <v>46043.385289351849</v>
       </c>
       <c r="F38" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G38" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H38" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I38" s="7">
         <v>1405794</v>
       </c>
       <c r="J38" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L38" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M38" s="10"/>
       <c r="N38" s="10">
@@ -2460,25 +2463,25 @@
         <v>46043.441296296296</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G39" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I39" s="7">
         <v>1405794</v>
       </c>
       <c r="J39" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L39" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M39" s="10"/>
       <c r="N39" s="10">
@@ -2501,25 +2504,25 @@
         <v>46044.570300925923</v>
       </c>
       <c r="F40" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G40" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H40" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I40" s="7">
         <v>1405794</v>
       </c>
       <c r="J40" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K40" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L40" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M40" s="10"/>
       <c r="N40" s="10">
@@ -2542,25 +2545,25 @@
         <v>46050.574884259258</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G41" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H41" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I41" s="7">
         <v>1411351</v>
       </c>
       <c r="J41" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K41" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L41" s="7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="M41" s="10"/>
       <c r="N41" s="10">
@@ -2583,25 +2586,25 @@
         <v>46051.280300925922</v>
       </c>
       <c r="F42" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G42" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H42" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I42" s="7">
         <v>1411352</v>
       </c>
       <c r="J42" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K42" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L42" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M42" s="10"/>
       <c r="N42" s="10">
@@ -2624,25 +2627,25 @@
         <v>46056.33489583333</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G43" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H43" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I43" s="7">
         <v>1410338</v>
       </c>
       <c r="J43" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K43" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L43" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M43" s="10"/>
       <c r="N43" s="10">
@@ -2665,25 +2668,25 @@
         <v>46062.345243055555</v>
       </c>
       <c r="F44" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G44" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H44" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I44" s="7">
         <v>1412987</v>
       </c>
       <c r="J44" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="K44" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L44" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M44" s="10"/>
       <c r="N44" s="10">
@@ -2706,25 +2709,25 @@
         <v>46064.292500000003</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G45" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H45" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I45" s="7">
         <v>1412987</v>
       </c>
       <c r="J45" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="K45" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L45" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M45" s="10"/>
       <c r="N45" s="10">
@@ -2747,25 +2750,25 @@
         <v>46073.402627314812</v>
       </c>
       <c r="F46" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G46" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H46" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I46" s="7">
         <v>1421099</v>
       </c>
       <c r="J46" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K46" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L46" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M46" s="10"/>
       <c r="N46" s="10">
@@ -2832,25 +2835,25 @@
         <v>46027.666331018518</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G49" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H49" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I49" s="7">
         <v>1386388</v>
       </c>
       <c r="J49" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K49" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L49" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M49" s="10"/>
       <c r="N49" s="10">
@@ -2873,25 +2876,25 @@
         <v>46027.694131944445</v>
       </c>
       <c r="F50" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G50" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H50" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I50" s="7">
         <v>1386388</v>
       </c>
       <c r="J50" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K50" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L50" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M50" s="10"/>
       <c r="N50" s="10">
@@ -2914,25 +2917,25 @@
         <v>46036.841574074075</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G51" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H51" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I51" s="7">
         <v>1406206</v>
       </c>
       <c r="J51" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K51" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L51" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="M51" s="10"/>
       <c r="N51" s="10">
@@ -2955,25 +2958,25 @@
         <v>46059.905682870369</v>
       </c>
       <c r="F52" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G52" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H52" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I52" s="7">
         <v>1411984</v>
       </c>
       <c r="J52" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K52" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L52" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="M52" s="10"/>
       <c r="N52" s="10">
@@ -2996,25 +2999,25 @@
         <v>46064.60796296296</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G53" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H53" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I53" s="7">
         <v>1411990</v>
       </c>
       <c r="J53" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="K53" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L53" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M53" s="10"/>
       <c r="N53" s="10">
@@ -3037,25 +3040,25 @@
         <v>46065.655185185184</v>
       </c>
       <c r="F54" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G54" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H54" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I54" s="7">
         <v>1411990</v>
       </c>
       <c r="J54" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="K54" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L54" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M54" s="10"/>
       <c r="N54" s="10">
@@ -3078,25 +3081,25 @@
         <v>46066.613657407404</v>
       </c>
       <c r="F55" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G55" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H55" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I55" s="7">
         <v>1411990</v>
       </c>
       <c r="J55" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="K55" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L55" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M55" s="10"/>
       <c r="N55" s="10">
@@ -3119,25 +3122,25 @@
         <v>46066.670127314814</v>
       </c>
       <c r="F56" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G56" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H56" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I56" s="7">
         <v>1411990</v>
       </c>
       <c r="J56" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="K56" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L56" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M56" s="10"/>
       <c r="N56" s="10">
@@ -3160,25 +3163,25 @@
         <v>46028.907905092594</v>
       </c>
       <c r="F57" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G57" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H57" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I57" s="7">
         <v>1394721</v>
       </c>
       <c r="J57" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K57" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L57" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M57" s="10"/>
       <c r="N57" s="10">
@@ -3201,25 +3204,25 @@
         <v>46029.6719212963</v>
       </c>
       <c r="F58" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G58" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H58" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I58" s="7">
         <v>1394721</v>
       </c>
       <c r="J58" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K58" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L58" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M58" s="10"/>
       <c r="N58" s="10">
@@ -3242,25 +3245,25 @@
         <v>46034.72855324074</v>
       </c>
       <c r="F59" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G59" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H59" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I59" s="7">
         <v>1394721</v>
       </c>
       <c r="J59" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K59" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L59" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M59" s="10"/>
       <c r="N59" s="10">
@@ -3283,25 +3286,25 @@
         <v>46037.838958333334</v>
       </c>
       <c r="F60" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G60" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H60" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I60" s="7">
         <v>1394721</v>
       </c>
       <c r="J60" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K60" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L60" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M60" s="10"/>
       <c r="N60" s="10">
@@ -3324,25 +3327,25 @@
         <v>46042.727754629632</v>
       </c>
       <c r="F61" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G61" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H61" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I61" s="7">
         <v>1394721</v>
       </c>
       <c r="J61" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K61" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L61" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M61" s="10"/>
       <c r="N61" s="10">
@@ -3365,25 +3368,25 @@
         <v>46043.627881944441</v>
       </c>
       <c r="F62" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G62" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H62" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I62" s="7">
         <v>1410339</v>
       </c>
       <c r="J62" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K62" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L62" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M62" s="10"/>
       <c r="N62" s="10">
@@ -3406,25 +3409,25 @@
         <v>46052.626018518517</v>
       </c>
       <c r="F63" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G63" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H63" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I63" s="7">
         <v>1411706</v>
       </c>
       <c r="J63" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K63" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L63" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="M63" s="10"/>
       <c r="N63" s="10">
@@ -3447,25 +3450,25 @@
         <v>46053.632291666669</v>
       </c>
       <c r="F64" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G64" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H64" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I64" s="7">
         <v>1411708</v>
       </c>
       <c r="J64" s="5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K64" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L64" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="M64" s="10"/>
       <c r="N64" s="10">
@@ -3488,25 +3491,25 @@
         <v>46071.601446759261</v>
       </c>
       <c r="F65" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G65" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H65" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I65" s="7">
         <v>1418251</v>
       </c>
       <c r="J65" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K65" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L65" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M65" s="10"/>
       <c r="N65" s="10">
@@ -3517,41 +3520,41 @@
     <row r="66" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A66" s="2"/>
       <c r="B66" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="D66" s="8">
-        <v>46027.633611111109</v>
+        <v>46076.679282407407</v>
       </c>
       <c r="E66" s="8">
-        <v>46027.633611111109</v>
+        <v>46076.679282407407</v>
       </c>
       <c r="F66" s="7" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G66" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H66" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I66" s="7">
-        <v>1404289</v>
+        <v>1422511</v>
       </c>
       <c r="J66" s="5" t="s">
         <v>79</v>
       </c>
       <c r="K66" s="5" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="L66" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M66" s="10"/>
       <c r="N66" s="10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O66" s="7"/>
     </row>
@@ -3561,38 +3564,38 @@
         <v>6</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="D67" s="8">
-        <v>46029.802372685182</v>
+        <v>46027.633611111109</v>
       </c>
       <c r="E67" s="8">
-        <v>46029.802372685182</v>
+        <v>46027.633611111109</v>
       </c>
       <c r="F67" s="7" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="G67" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H67" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I67" s="7">
-        <v>1394724</v>
+        <v>1404289</v>
       </c>
       <c r="J67" s="5" t="s">
         <v>80</v>
       </c>
       <c r="K67" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L67" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M67" s="10"/>
       <c r="N67" s="10">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="O67" s="7"/>
     </row>
@@ -3602,19 +3605,19 @@
         <v>6</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="D68" s="8">
-        <v>46030.908472222225</v>
+        <v>46029.802372685182</v>
       </c>
       <c r="E68" s="8">
-        <v>46030.908472222225</v>
+        <v>46029.802372685182</v>
       </c>
       <c r="F68" s="7" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G68" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H68" s="5" t="s">
         <v>66</v>
@@ -3623,17 +3626,17 @@
         <v>1394724</v>
       </c>
       <c r="J68" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K68" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L68" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M68" s="10"/>
       <c r="N68" s="10">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="O68" s="7"/>
     </row>
@@ -3643,120 +3646,120 @@
         <v>6</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D69" s="8">
-        <v>46031.590057870373</v>
+        <v>46030.908472222225</v>
       </c>
       <c r="E69" s="8">
-        <v>46031.590057870373</v>
+        <v>46030.908472222225</v>
       </c>
       <c r="F69" s="7" t="s">
         <v>57</v>
       </c>
       <c r="G69" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H69" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I69" s="7">
         <v>1394724</v>
       </c>
       <c r="J69" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K69" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L69" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M69" s="10"/>
       <c r="N69" s="10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O69" s="7"/>
     </row>
     <row r="70" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A70" s="2"/>
       <c r="B70" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="D70" s="8">
-        <v>46024.795127314814</v>
+        <v>46031.590057870373</v>
       </c>
       <c r="E70" s="8">
-        <v>46024.795127314814</v>
+        <v>46031.590057870373</v>
       </c>
       <c r="F70" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G70" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H70" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I70" s="7">
-        <v>1398335</v>
+        <v>1394724</v>
       </c>
       <c r="J70" s="5" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="K70" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L70" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M70" s="10"/>
       <c r="N70" s="10">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O70" s="7"/>
     </row>
     <row r="71" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A71" s="2"/>
       <c r="B71" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C71" s="7" t="s">
         <v>40</v>
       </c>
       <c r="D71" s="8">
-        <v>46024.795277777775</v>
+        <v>46076.8827662037</v>
       </c>
       <c r="E71" s="8">
-        <v>46024.795277777775</v>
+        <v>46076.8827662037</v>
       </c>
       <c r="F71" s="7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G71" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H71" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I71" s="7">
-        <v>1398335</v>
+        <v>1422286</v>
       </c>
       <c r="J71" s="5" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="K71" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L71" s="7" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="M71" s="10"/>
       <c r="N71" s="10">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="O71" s="7"/>
     </row>
@@ -3766,38 +3769,38 @@
         <v>7</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D72" s="8">
-        <v>46024.900324074071</v>
+        <v>46024.795127314814</v>
       </c>
       <c r="E72" s="8">
-        <v>46024.900324074071</v>
+        <v>46024.795127314814</v>
       </c>
       <c r="F72" s="7" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G72" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H72" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I72" s="7">
         <v>1398335</v>
       </c>
       <c r="J72" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="K72" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L72" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M72" s="10"/>
       <c r="N72" s="10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O72" s="7"/>
     </row>
@@ -3807,34 +3810,34 @@
         <v>7</v>
       </c>
       <c r="C73" s="7" t="s">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="D73" s="8">
-        <v>46028.866898148146</v>
+        <v>46024.795277777775</v>
       </c>
       <c r="E73" s="8">
-        <v>46028.866898148146</v>
+        <v>46024.795277777775</v>
       </c>
       <c r="F73" s="7" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="G73" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H73" s="5" t="s">
         <v>66</v>
       </c>
       <c r="I73" s="7">
-        <v>1402956</v>
+        <v>1398335</v>
       </c>
       <c r="J73" s="5" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="K73" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L73" s="7" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="M73" s="10"/>
       <c r="N73" s="10">
@@ -3848,38 +3851,38 @@
         <v>7</v>
       </c>
       <c r="C74" s="7" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D74" s="8">
-        <v>46034.751261574071</v>
+        <v>46024.900324074071</v>
       </c>
       <c r="E74" s="8">
-        <v>46034.751261574071</v>
+        <v>46024.900324074071</v>
       </c>
       <c r="F74" s="7" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="G74" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H74" s="5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I74" s="7">
-        <v>1404958</v>
+        <v>1398335</v>
       </c>
       <c r="J74" s="5" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="K74" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L74" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M74" s="10"/>
       <c r="N74" s="10">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O74" s="7"/>
     </row>
@@ -3889,38 +3892,38 @@
         <v>7</v>
       </c>
       <c r="C75" s="7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D75" s="8">
-        <v>46062.904895833337</v>
+        <v>46028.866898148146</v>
       </c>
       <c r="E75" s="8">
-        <v>46062.904895833337</v>
+        <v>46028.866898148146</v>
       </c>
       <c r="F75" s="7" t="s">
         <v>56</v>
       </c>
       <c r="G75" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H75" s="5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I75" s="7">
-        <v>1412987</v>
+        <v>1402956</v>
       </c>
       <c r="J75" s="5" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="K75" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L75" s="7" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="M75" s="10"/>
       <c r="N75" s="10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O75" s="7"/>
     </row>
@@ -3930,38 +3933,38 @@
         <v>7</v>
       </c>
       <c r="C76" s="7" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="D76" s="8">
-        <v>46063.874467592592</v>
+        <v>46034.751261574071</v>
       </c>
       <c r="E76" s="8">
-        <v>46063.874467592592</v>
+        <v>46034.751261574071</v>
       </c>
       <c r="F76" s="7" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="G76" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H76" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I76" s="7">
-        <v>1412987</v>
+        <v>1404958</v>
       </c>
       <c r="J76" s="5" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="K76" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L76" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M76" s="10"/>
       <c r="N76" s="10">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="O76" s="7"/>
     </row>
@@ -3971,38 +3974,38 @@
         <v>7</v>
       </c>
       <c r="C77" s="7" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="D77" s="8">
-        <v>46067.906875000001</v>
+        <v>46062.904895833337</v>
       </c>
       <c r="E77" s="8">
-        <v>46067.906875000001</v>
+        <v>46062.904895833337</v>
       </c>
       <c r="F77" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G77" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H77" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I77" s="7">
-        <v>1411991</v>
+        <v>1412987</v>
       </c>
       <c r="J77" s="5" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="K77" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L77" s="7" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="M77" s="10"/>
       <c r="N77" s="10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O77" s="7"/>
     </row>
@@ -4012,87 +4015,169 @@
         <v>7</v>
       </c>
       <c r="C78" s="7" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="D78" s="8">
-        <v>46069.700543981482</v>
+        <v>46063.874467592592</v>
       </c>
       <c r="E78" s="8">
-        <v>46069.700543981482</v>
+        <v>46063.874467592592</v>
       </c>
       <c r="F78" s="7" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G78" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H78" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I78" s="7">
-        <v>1411991</v>
+        <v>1412987</v>
       </c>
       <c r="J78" s="5" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="K78" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L78" s="7" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="M78" s="10"/>
       <c r="N78" s="10">
+        <v>5</v>
+      </c>
+      <c r="O78" s="7"/>
+    </row>
+    <row r="79" spans="1:15" ht="21" x14ac:dyDescent="0.2">
+      <c r="A79" s="2"/>
+      <c r="B79" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C79" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D79" s="8">
+        <v>46067.906875000001</v>
+      </c>
+      <c r="E79" s="8">
+        <v>46067.906875000001</v>
+      </c>
+      <c r="F79" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="G79" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="H79" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="I79" s="7">
+        <v>1411991</v>
+      </c>
+      <c r="J79" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="K79" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="L79" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="M79" s="10"/>
+      <c r="N79" s="10">
+        <v>3</v>
+      </c>
+      <c r="O79" s="7"/>
+    </row>
+    <row r="80" spans="1:15" ht="21" x14ac:dyDescent="0.2">
+      <c r="A80" s="2"/>
+      <c r="B80" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C80" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D80" s="8">
+        <v>46069.700543981482</v>
+      </c>
+      <c r="E80" s="8">
+        <v>46069.700543981482</v>
+      </c>
+      <c r="F80" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="G80" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="H80" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="I80" s="7">
+        <v>1411991</v>
+      </c>
+      <c r="J80" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="K80" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="L80" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="M80" s="10"/>
+      <c r="N80" s="10">
         <v>10</v>
       </c>
-      <c r="O78" s="7"/>
-    </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A79" s="4"/>
-      <c r="B79" s="6"/>
-      <c r="C79" s="6"/>
-      <c r="D79" s="6"/>
-      <c r="E79" s="6"/>
-      <c r="F79" s="6"/>
-      <c r="G79" s="6"/>
-      <c r="H79" s="6"/>
-      <c r="I79" s="6"/>
-      <c r="J79" s="6"/>
-      <c r="K79" s="6"/>
-      <c r="L79" s="6"/>
-      <c r="M79" s="9">
+      <c r="O80" s="7"/>
+    </row>
+    <row r="81" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A81" s="4"/>
+      <c r="B81" s="6"/>
+      <c r="C81" s="6"/>
+      <c r="D81" s="6"/>
+      <c r="E81" s="6"/>
+      <c r="F81" s="6"/>
+      <c r="G81" s="6"/>
+      <c r="H81" s="6"/>
+      <c r="I81" s="6"/>
+      <c r="J81" s="6"/>
+      <c r="K81" s="6"/>
+      <c r="L81" s="6"/>
+      <c r="M81" s="9">
         <v>0</v>
       </c>
-      <c r="N79" s="9">
-        <v>144</v>
-      </c>
-      <c r="O79" s="9">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A80" s="4"/>
-      <c r="B80" s="6"/>
-      <c r="C80" s="6"/>
-      <c r="D80" s="6"/>
-      <c r="E80" s="6"/>
-      <c r="F80" s="6"/>
-      <c r="G80" s="6"/>
-      <c r="H80" s="9">
-        <v>73</v>
-      </c>
-      <c r="I80" s="6"/>
-      <c r="J80" s="6"/>
-      <c r="K80" s="6"/>
-      <c r="L80" s="6"/>
-      <c r="M80" s="9">
+      <c r="N81" s="9">
+        <v>160</v>
+      </c>
+      <c r="O81" s="9">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="82" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A82" s="4"/>
+      <c r="B82" s="6"/>
+      <c r="C82" s="6"/>
+      <c r="D82" s="6"/>
+      <c r="E82" s="6"/>
+      <c r="F82" s="6"/>
+      <c r="G82" s="6"/>
+      <c r="H82" s="9">
+        <v>75</v>
+      </c>
+      <c r="I82" s="6"/>
+      <c r="J82" s="6"/>
+      <c r="K82" s="6"/>
+      <c r="L82" s="6"/>
+      <c r="M82" s="9">
         <v>0</v>
       </c>
-      <c r="N80" s="9">
-        <v>339</v>
-      </c>
-      <c r="O80" s="9">
-        <v>73</v>
+      <c r="N82" s="9">
+        <v>355</v>
+      </c>
+      <c r="O82" s="9">
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica (25/02/2026  8:15:08,63)
</commit_message>
<xml_diff>
--- a/rejeito.xlsx
+++ b/rejeito.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PLANILHAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{798F27DA-7352-4B62-8567-053B09BACDB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AF00A9EC-A8C0-41AA-8345-FC909CFD9F35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3585" yWindow="3585" windowWidth="21600" windowHeight="11295" xr2:uid="{07B4FCB3-FF16-4E63-8B27-07285E70AFC4}"/>
+    <workbookView xWindow="3930" yWindow="3930" windowWidth="21600" windowHeight="11295" xr2:uid="{F406952C-5FB2-4B25-BBFE-996FA6F356DB}"/>
   </bookViews>
   <sheets>
     <sheet name="rejeito" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="669" uniqueCount="114">
   <si>
     <t>Dados</t>
   </si>
@@ -95,6 +95,9 @@
   </si>
   <si>
     <t>20/02/2026</t>
+  </si>
+  <si>
+    <t>24/02/2026</t>
   </si>
   <si>
     <t>05/01/2026</t>
@@ -903,8 +906,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3CA8AB7-A591-4CD1-85BC-46C85D7EFCC6}">
-  <dimension ref="A1:O82"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9ADE1002-6B5E-4CC2-89CC-99B3A2A3AACB}">
+  <dimension ref="A1:O88"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.42578125" customWidth="1"/>
@@ -935,14 +938,14 @@
       <c r="F1" s="11"/>
       <c r="G1" s="11"/>
       <c r="H1" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I1" s="11"/>
       <c r="J1" s="11"/>
       <c r="K1" s="11"/>
       <c r="L1" s="11"/>
       <c r="M1" s="11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="N1" s="11"/>
       <c r="O1" s="11"/>
@@ -956,40 +959,40 @@
         <v>9</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:15" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1028,25 +1031,25 @@
         <v>46046.443344907406</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I4" s="7">
         <v>1406207</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M4" s="10"/>
       <c r="N4" s="10">
@@ -1069,25 +1072,25 @@
         <v>46046.553217592591</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I5" s="7">
         <v>1406207</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M5" s="10"/>
       <c r="N5" s="10">
@@ -1110,25 +1113,25 @@
         <v>46050.493333333332</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I6" s="7">
         <v>1411349</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L6" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="M6" s="10"/>
       <c r="N6" s="10">
@@ -1151,25 +1154,25 @@
         <v>46051.555428240739</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I7" s="7">
         <v>1411348</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="M7" s="10"/>
       <c r="N7" s="10">
@@ -1192,25 +1195,25 @@
         <v>46053.377129629633</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I8" s="7">
         <v>1409954</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M8" s="10"/>
       <c r="N8" s="10">
@@ -1233,25 +1236,25 @@
         <v>46062.302418981482</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I9" s="7">
         <v>1411984</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L9" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="M9" s="10"/>
       <c r="N9" s="10">
@@ -1274,25 +1277,25 @@
         <v>46062.570879629631</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I10" s="7">
         <v>1411984</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="M10" s="10"/>
       <c r="N10" s="10">
@@ -1315,25 +1318,25 @@
         <v>46064.297777777778</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I11" s="7">
         <v>1411984</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L11" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="M11" s="10"/>
       <c r="N11" s="10">
@@ -1356,25 +1359,25 @@
         <v>46064.455104166664</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I12" s="7">
         <v>1411990</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="M12" s="10"/>
       <c r="N12" s="10">
@@ -1397,25 +1400,25 @@
         <v>46028.331469907411</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I13" s="7">
         <v>1402958</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L13" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M13" s="10"/>
       <c r="N13" s="10">
@@ -1438,25 +1441,25 @@
         <v>46030.306192129632</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I14" s="7">
         <v>1394721</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L14" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M14" s="10"/>
       <c r="N14" s="10">
@@ -1479,25 +1482,25 @@
         <v>46031.443101851852</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I15" s="7">
         <v>1394721</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M15" s="10"/>
       <c r="N15" s="10">
@@ -1520,25 +1523,25 @@
         <v>46035.530381944445</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I16" s="7">
         <v>1394721</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L16" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M16" s="10"/>
       <c r="N16" s="10">
@@ -1561,25 +1564,25 @@
         <v>46046.391701388886</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I17" s="7">
         <v>1410340</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L17" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M17" s="10"/>
       <c r="N17" s="10">
@@ -1602,25 +1605,25 @@
         <v>46046.516597222224</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I18" s="7">
         <v>1410340</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L18" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M18" s="10"/>
       <c r="N18" s="10">
@@ -1643,25 +1646,25 @@
         <v>46048.278912037036</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I19" s="7">
         <v>1410340</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K19" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L19" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M19" s="10"/>
       <c r="N19" s="10">
@@ -1684,25 +1687,25 @@
         <v>46051.403391203705</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I20" s="7">
         <v>1410340</v>
       </c>
       <c r="J20" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K20" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L20" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M20" s="10"/>
       <c r="N20" s="10">
@@ -1725,25 +1728,25 @@
         <v>46053.550381944442</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I21" s="7">
         <v>1411706</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L21" s="7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="M21" s="10"/>
       <c r="N21" s="10">
@@ -1766,25 +1769,25 @@
         <v>46057.413171296299</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I22" s="7">
         <v>1411704</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L22" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M22" s="10"/>
       <c r="N22" s="10">
@@ -1807,25 +1810,25 @@
         <v>46058.357476851852</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I23" s="7">
         <v>1411704</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L23" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M23" s="10"/>
       <c r="N23" s="10">
@@ -1848,25 +1851,25 @@
         <v>46058.531793981485</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I24" s="7">
         <v>1411704</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L24" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M24" s="10"/>
       <c r="N24" s="10">
@@ -1889,25 +1892,25 @@
         <v>46067.433020833334</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I25" s="7">
         <v>1418256</v>
       </c>
       <c r="J25" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L25" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M25" s="10"/>
       <c r="N25" s="10">
@@ -1930,25 +1933,25 @@
         <v>46073.579664351855</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I26" s="7">
         <v>1422511</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L26" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M26" s="10"/>
       <c r="N26" s="10">
@@ -1959,28 +1962,28 @@
     <row r="27" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A27" s="2"/>
       <c r="B27" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C27" s="7" t="s">
         <v>25</v>
       </c>
       <c r="D27" s="8">
-        <v>46027.4840625</v>
+        <v>46077.38318287037</v>
       </c>
       <c r="E27" s="8">
-        <v>46027.4840625</v>
+        <v>46077.38318287037</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I27" s="7">
-        <v>1404289</v>
+        <v>1422511</v>
       </c>
       <c r="J27" s="5" t="s">
         <v>80</v>
@@ -1989,11 +1992,11 @@
         <v>97</v>
       </c>
       <c r="L27" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M27" s="10"/>
       <c r="N27" s="10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O27" s="7"/>
     </row>
@@ -2003,38 +2006,38 @@
         <v>6</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="D28" s="8">
-        <v>46030.397997685184</v>
+        <v>46027.4840625</v>
       </c>
       <c r="E28" s="8">
-        <v>46030.397997685184</v>
+        <v>46027.4840625</v>
       </c>
       <c r="F28" s="7" t="s">
         <v>49</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I28" s="7">
-        <v>1394724</v>
+        <v>1404289</v>
       </c>
       <c r="J28" s="5" t="s">
         <v>81</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L28" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M28" s="10"/>
       <c r="N28" s="10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O28" s="7"/>
     </row>
@@ -2047,31 +2050,31 @@
         <v>17</v>
       </c>
       <c r="D29" s="8">
-        <v>46030.408148148148</v>
+        <v>46030.397997685184</v>
       </c>
       <c r="E29" s="8">
-        <v>46030.408148148148</v>
+        <v>46030.397997685184</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I29" s="7">
         <v>1394724</v>
       </c>
       <c r="J29" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L29" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M29" s="10"/>
       <c r="N29" s="10">
@@ -2088,31 +2091,31 @@
         <v>17</v>
       </c>
       <c r="D30" s="8">
-        <v>46030.478854166664</v>
+        <v>46030.408148148148</v>
       </c>
       <c r="E30" s="8">
-        <v>46030.478854166664</v>
+        <v>46030.408148148148</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G30" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I30" s="7">
         <v>1394724</v>
       </c>
       <c r="J30" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L30" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M30" s="10"/>
       <c r="N30" s="10">
@@ -2129,35 +2132,35 @@
         <v>17</v>
       </c>
       <c r="D31" s="8">
-        <v>46030.561284722222</v>
+        <v>46030.478854166664</v>
       </c>
       <c r="E31" s="8">
-        <v>46030.561284722222</v>
+        <v>46030.478854166664</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G31" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I31" s="7">
         <v>1394724</v>
       </c>
       <c r="J31" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L31" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M31" s="10"/>
       <c r="N31" s="10">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O31" s="7"/>
     </row>
@@ -2167,38 +2170,38 @@
         <v>6</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D32" s="8">
-        <v>46035.478368055556</v>
+        <v>46030.561284722222</v>
       </c>
       <c r="E32" s="8">
-        <v>46035.478368055556</v>
+        <v>46030.561284722222</v>
       </c>
       <c r="F32" s="7" t="s">
         <v>48</v>
       </c>
       <c r="G32" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I32" s="7">
         <v>1394724</v>
       </c>
       <c r="J32" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L32" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M32" s="10"/>
       <c r="N32" s="10">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="O32" s="7"/>
     </row>
@@ -2208,38 +2211,38 @@
         <v>6</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="D33" s="8">
-        <v>46043.385474537034</v>
+        <v>46035.478368055556</v>
       </c>
       <c r="E33" s="8">
-        <v>46043.385474537034</v>
+        <v>46035.478368055556</v>
       </c>
       <c r="F33" s="7" t="s">
         <v>49</v>
       </c>
       <c r="G33" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I33" s="7">
         <v>1394724</v>
       </c>
       <c r="J33" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L33" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M33" s="10"/>
       <c r="N33" s="10">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="O33" s="7"/>
     </row>
@@ -2249,34 +2252,34 @@
         <v>6</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D34" s="8">
-        <v>46043.565196759257</v>
+        <v>46043.385474537034</v>
       </c>
       <c r="E34" s="8">
-        <v>46043.565196759257</v>
+        <v>46043.385474537034</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G34" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I34" s="7">
         <v>1394724</v>
       </c>
       <c r="J34" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="L34" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M34" s="10"/>
       <c r="N34" s="10">
@@ -2293,22 +2296,22 @@
         <v>27</v>
       </c>
       <c r="D35" s="8">
-        <v>46069.559953703705</v>
+        <v>46043.565196759257</v>
       </c>
       <c r="E35" s="8">
-        <v>46069.559953703705</v>
+        <v>46043.565196759257</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G35" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I35" s="7">
-        <v>1421099</v>
+        <v>1394724</v>
       </c>
       <c r="J35" s="5" t="s">
         <v>82</v>
@@ -2317,52 +2320,52 @@
         <v>97</v>
       </c>
       <c r="L35" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M35" s="10"/>
       <c r="N35" s="10">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O35" s="7"/>
     </row>
     <row r="36" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
       <c r="B36" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="D36" s="8">
-        <v>46035.47824074074</v>
+        <v>46069.559953703705</v>
       </c>
       <c r="E36" s="8">
-        <v>46035.47824074074</v>
+        <v>46069.559953703705</v>
       </c>
       <c r="F36" s="7" t="s">
         <v>48</v>
       </c>
       <c r="G36" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H36" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I36" s="7">
-        <v>1404958</v>
+        <v>1421099</v>
       </c>
       <c r="J36" s="5" t="s">
         <v>83</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L36" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M36" s="10"/>
       <c r="N36" s="10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O36" s="7"/>
     </row>
@@ -2372,38 +2375,38 @@
         <v>7</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="D37" s="8">
-        <v>46043.385196759256</v>
+        <v>46035.47824074074</v>
       </c>
       <c r="E37" s="8">
-        <v>46043.385196759256</v>
+        <v>46035.47824074074</v>
       </c>
       <c r="F37" s="7" t="s">
         <v>49</v>
       </c>
       <c r="G37" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H37" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I37" s="7">
-        <v>1405794</v>
+        <v>1404958</v>
       </c>
       <c r="J37" s="5" t="s">
         <v>84</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L37" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M37" s="10"/>
       <c r="N37" s="10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O37" s="7"/>
     </row>
@@ -2413,19 +2416,19 @@
         <v>7</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D38" s="8">
-        <v>46043.385289351849</v>
+        <v>46043.385196759256</v>
       </c>
       <c r="E38" s="8">
-        <v>46043.385289351849</v>
+        <v>46043.385196759256</v>
       </c>
       <c r="F38" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G38" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H38" s="5" t="s">
         <v>67</v>
@@ -2434,17 +2437,17 @@
         <v>1405794</v>
       </c>
       <c r="J38" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L38" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M38" s="10"/>
       <c r="N38" s="10">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O38" s="7"/>
     </row>
@@ -2454,38 +2457,38 @@
         <v>7</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D39" s="8">
-        <v>46043.441296296296</v>
+        <v>46043.385289351849</v>
       </c>
       <c r="E39" s="8">
-        <v>46043.441296296296</v>
+        <v>46043.385289351849</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="G39" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I39" s="7">
         <v>1405794</v>
       </c>
       <c r="J39" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L39" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M39" s="10"/>
       <c r="N39" s="10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O39" s="7"/>
     </row>
@@ -2495,38 +2498,38 @@
         <v>7</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D40" s="8">
-        <v>46044.570300925923</v>
+        <v>46043.441296296296</v>
       </c>
       <c r="E40" s="8">
-        <v>46044.570300925923</v>
+        <v>46043.441296296296</v>
       </c>
       <c r="F40" s="7" t="s">
         <v>47</v>
       </c>
       <c r="G40" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H40" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I40" s="7">
         <v>1405794</v>
       </c>
       <c r="J40" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K40" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L40" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M40" s="10"/>
       <c r="N40" s="10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O40" s="7"/>
     </row>
@@ -2536,38 +2539,38 @@
         <v>7</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="D41" s="8">
-        <v>46050.574884259258</v>
+        <v>46044.570300925923</v>
       </c>
       <c r="E41" s="8">
-        <v>46050.574884259258</v>
+        <v>46044.570300925923</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G41" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H41" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I41" s="7">
-        <v>1411351</v>
+        <v>1405794</v>
       </c>
       <c r="J41" s="5" t="s">
         <v>85</v>
       </c>
       <c r="K41" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L41" s="7" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="M41" s="10"/>
       <c r="N41" s="10">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="O41" s="7"/>
     </row>
@@ -2577,38 +2580,38 @@
         <v>7</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D42" s="8">
-        <v>46051.280300925922</v>
+        <v>46050.574884259258</v>
       </c>
       <c r="E42" s="8">
-        <v>46051.280300925922</v>
+        <v>46050.574884259258</v>
       </c>
       <c r="F42" s="7" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="G42" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H42" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I42" s="7">
-        <v>1411352</v>
+        <v>1411351</v>
       </c>
       <c r="J42" s="5" t="s">
         <v>86</v>
       </c>
       <c r="K42" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L42" s="7" t="s">
         <v>106</v>
       </c>
       <c r="M42" s="10"/>
       <c r="N42" s="10">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="O42" s="7"/>
     </row>
@@ -2618,38 +2621,38 @@
         <v>7</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="D43" s="8">
-        <v>46056.33489583333</v>
+        <v>46051.280300925922</v>
       </c>
       <c r="E43" s="8">
-        <v>46056.33489583333</v>
+        <v>46051.280300925922</v>
       </c>
       <c r="F43" s="7" t="s">
         <v>53</v>
       </c>
       <c r="G43" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H43" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I43" s="7">
-        <v>1410338</v>
+        <v>1411352</v>
       </c>
       <c r="J43" s="5" t="s">
         <v>87</v>
       </c>
       <c r="K43" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L43" s="7" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="M43" s="10"/>
       <c r="N43" s="10">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="O43" s="7"/>
     </row>
@@ -2659,38 +2662,38 @@
         <v>7</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="D44" s="8">
-        <v>46062.345243055555</v>
+        <v>46056.33489583333</v>
       </c>
       <c r="E44" s="8">
-        <v>46062.345243055555</v>
+        <v>46056.33489583333</v>
       </c>
       <c r="F44" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G44" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H44" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I44" s="7">
-        <v>1412987</v>
+        <v>1410338</v>
       </c>
       <c r="J44" s="5" t="s">
         <v>88</v>
       </c>
       <c r="K44" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L44" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M44" s="10"/>
       <c r="N44" s="10">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="O44" s="7"/>
     </row>
@@ -2700,38 +2703,38 @@
         <v>7</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D45" s="8">
-        <v>46064.292500000003</v>
+        <v>46062.345243055555</v>
       </c>
       <c r="E45" s="8">
-        <v>46064.292500000003</v>
+        <v>46062.345243055555</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G45" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H45" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I45" s="7">
         <v>1412987</v>
       </c>
       <c r="J45" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K45" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L45" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M45" s="10"/>
       <c r="N45" s="10">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="O45" s="7"/>
     </row>
@@ -2741,119 +2744,157 @@
         <v>7</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="D46" s="8">
-        <v>46073.402627314812</v>
+        <v>46064.292500000003</v>
       </c>
       <c r="E46" s="8">
-        <v>46073.402627314812</v>
+        <v>46064.292500000003</v>
       </c>
       <c r="F46" s="7" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G46" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H46" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I46" s="7">
-        <v>1421099</v>
+        <v>1412987</v>
       </c>
       <c r="J46" s="5" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="K46" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L46" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M46" s="10"/>
       <c r="N46" s="10">
+        <v>3</v>
+      </c>
+      <c r="O46" s="7"/>
+    </row>
+    <row r="47" spans="1:15" ht="21" x14ac:dyDescent="0.2">
+      <c r="A47" s="2"/>
+      <c r="B47" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D47" s="8">
+        <v>46073.402627314812</v>
+      </c>
+      <c r="E47" s="8">
+        <v>46073.402627314812</v>
+      </c>
+      <c r="F47" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G47" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="H47" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="I47" s="7">
+        <v>1421099</v>
+      </c>
+      <c r="J47" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="K47" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="L47" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="M47" s="10"/>
+      <c r="N47" s="10">
         <v>2</v>
       </c>
-      <c r="O46" s="7"/>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A47" s="4"/>
-      <c r="B47" s="6"/>
-      <c r="C47" s="6"/>
-      <c r="D47" s="6"/>
-      <c r="E47" s="6"/>
-      <c r="F47" s="6"/>
-      <c r="G47" s="6"/>
-      <c r="H47" s="6"/>
-      <c r="I47" s="6"/>
-      <c r="J47" s="6"/>
-      <c r="K47" s="6"/>
-      <c r="L47" s="6"/>
-      <c r="M47" s="9">
-        <v>0</v>
-      </c>
-      <c r="N47" s="9">
-        <v>195</v>
-      </c>
-      <c r="O47" s="9">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="48" spans="1:15" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B48" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="C48" s="12"/>
-      <c r="D48" s="12"/>
-      <c r="E48" s="12"/>
-      <c r="F48" s="12"/>
-      <c r="G48" s="12"/>
-      <c r="H48" s="12"/>
-      <c r="I48" s="12"/>
-      <c r="J48" s="12"/>
-      <c r="K48" s="12"/>
-      <c r="L48" s="12"/>
-      <c r="M48" s="12"/>
-      <c r="N48" s="12"/>
-      <c r="O48" s="12"/>
+      <c r="O47" s="7"/>
+    </row>
+    <row r="48" spans="1:15" ht="21" x14ac:dyDescent="0.2">
+      <c r="A48" s="2"/>
+      <c r="B48" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C48" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D48" s="8">
+        <v>46077.368379629632</v>
+      </c>
+      <c r="E48" s="8">
+        <v>46077.368379629632</v>
+      </c>
+      <c r="F48" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="G48" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="H48" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="I48" s="7">
+        <v>1422285</v>
+      </c>
+      <c r="J48" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="K48" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="L48" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="M48" s="10"/>
+      <c r="N48" s="10">
+        <v>3</v>
+      </c>
+      <c r="O48" s="7"/>
     </row>
     <row r="49" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A49" s="2"/>
       <c r="B49" s="5" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C49" s="7" t="s">
         <v>25</v>
       </c>
       <c r="D49" s="8">
-        <v>46027.666331018518</v>
+        <v>46077.554594907408</v>
       </c>
       <c r="E49" s="8">
-        <v>46027.666331018518</v>
+        <v>46077.554594907408</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="G49" s="7" t="s">
         <v>64</v>
       </c>
       <c r="H49" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I49" s="7">
-        <v>1386388</v>
+        <v>1422285</v>
       </c>
       <c r="J49" s="5" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="K49" s="5" t="s">
         <v>98</v>
       </c>
       <c r="L49" s="7" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="M49" s="10"/>
       <c r="N49" s="10">
@@ -2861,87 +2902,49 @@
       </c>
       <c r="O49" s="7"/>
     </row>
-    <row r="50" spans="1:15" ht="21" x14ac:dyDescent="0.2">
-      <c r="A50" s="2"/>
-      <c r="B50" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C50" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="D50" s="8">
-        <v>46027.694131944445</v>
-      </c>
-      <c r="E50" s="8">
-        <v>46027.694131944445</v>
-      </c>
-      <c r="F50" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="G50" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="H50" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="I50" s="7">
-        <v>1386388</v>
-      </c>
-      <c r="J50" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="K50" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="L50" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="M50" s="10"/>
-      <c r="N50" s="10">
-        <v>1</v>
-      </c>
-      <c r="O50" s="7"/>
-    </row>
-    <row r="51" spans="1:15" ht="21" x14ac:dyDescent="0.2">
-      <c r="A51" s="2"/>
-      <c r="B51" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C51" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="D51" s="8">
-        <v>46036.841574074075</v>
-      </c>
-      <c r="E51" s="8">
-        <v>46036.841574074075</v>
-      </c>
-      <c r="F51" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="G51" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="H51" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="I51" s="7">
-        <v>1406206</v>
-      </c>
-      <c r="J51" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="K51" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="L51" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="M51" s="10"/>
-      <c r="N51" s="10">
-        <v>11</v>
-      </c>
-      <c r="O51" s="7"/>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A50" s="4"/>
+      <c r="B50" s="6"/>
+      <c r="C50" s="6"/>
+      <c r="D50" s="6"/>
+      <c r="E50" s="6"/>
+      <c r="F50" s="6"/>
+      <c r="G50" s="6"/>
+      <c r="H50" s="6"/>
+      <c r="I50" s="6"/>
+      <c r="J50" s="6"/>
+      <c r="K50" s="6"/>
+      <c r="L50" s="6"/>
+      <c r="M50" s="9">
+        <v>0</v>
+      </c>
+      <c r="N50" s="9">
+        <v>203</v>
+      </c>
+      <c r="O50" s="9">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="51" spans="1:15" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B51" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="C51" s="12"/>
+      <c r="D51" s="12"/>
+      <c r="E51" s="12"/>
+      <c r="F51" s="12"/>
+      <c r="G51" s="12"/>
+      <c r="H51" s="12"/>
+      <c r="I51" s="12"/>
+      <c r="J51" s="12"/>
+      <c r="K51" s="12"/>
+      <c r="L51" s="12"/>
+      <c r="M51" s="12"/>
+      <c r="N51" s="12"/>
+      <c r="O51" s="12"/>
     </row>
     <row r="52" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A52" s="2"/>
@@ -2949,38 +2952,38 @@
         <v>4</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="D52" s="8">
-        <v>46059.905682870369</v>
+        <v>46027.666331018518</v>
       </c>
       <c r="E52" s="8">
-        <v>46059.905682870369</v>
+        <v>46027.666331018518</v>
       </c>
       <c r="F52" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G52" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H52" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I52" s="7">
-        <v>1411984</v>
+        <v>1386388</v>
       </c>
       <c r="J52" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K52" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L52" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="M52" s="10"/>
       <c r="N52" s="10">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="O52" s="7"/>
     </row>
@@ -2990,38 +2993,38 @@
         <v>4</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="D53" s="8">
-        <v>46064.60796296296</v>
+        <v>46027.694131944445</v>
       </c>
       <c r="E53" s="8">
-        <v>46064.60796296296</v>
+        <v>46027.694131944445</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G53" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H53" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I53" s="7">
-        <v>1411990</v>
+        <v>1386388</v>
       </c>
       <c r="J53" s="5" t="s">
         <v>71</v>
       </c>
       <c r="K53" s="5" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="L53" s="7" t="s">
         <v>102</v>
       </c>
       <c r="M53" s="10"/>
       <c r="N53" s="10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O53" s="7"/>
     </row>
@@ -3031,38 +3034,38 @@
         <v>4</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D54" s="8">
-        <v>46065.655185185184</v>
+        <v>46036.841574074075</v>
       </c>
       <c r="E54" s="8">
-        <v>46065.655185185184</v>
+        <v>46036.841574074075</v>
       </c>
       <c r="F54" s="7" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="G54" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H54" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I54" s="7">
-        <v>1411990</v>
+        <v>1406206</v>
       </c>
       <c r="J54" s="5" t="s">
-        <v>71</v>
+        <v>90</v>
       </c>
       <c r="K54" s="5" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="L54" s="7" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="M54" s="10"/>
       <c r="N54" s="10">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="O54" s="7"/>
     </row>
@@ -3072,38 +3075,38 @@
         <v>4</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D55" s="8">
-        <v>46066.613657407404</v>
+        <v>46059.905682870369</v>
       </c>
       <c r="E55" s="8">
-        <v>46066.613657407404</v>
+        <v>46059.905682870369</v>
       </c>
       <c r="F55" s="7" t="s">
         <v>58</v>
       </c>
       <c r="G55" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H55" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I55" s="7">
-        <v>1411990</v>
+        <v>1411984</v>
       </c>
       <c r="J55" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K55" s="5" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="L55" s="7" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="M55" s="10"/>
       <c r="N55" s="10">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="O55" s="7"/>
     </row>
@@ -3113,34 +3116,34 @@
         <v>4</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="D56" s="8">
-        <v>46066.670127314814</v>
+        <v>46064.60796296296</v>
       </c>
       <c r="E56" s="8">
-        <v>46066.670127314814</v>
+        <v>46064.60796296296</v>
       </c>
       <c r="F56" s="7" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G56" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H56" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I56" s="7">
         <v>1411990</v>
       </c>
       <c r="J56" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K56" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L56" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="M56" s="10"/>
       <c r="N56" s="10">
@@ -3151,123 +3154,123 @@
     <row r="57" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A57" s="2"/>
       <c r="B57" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="D57" s="8">
-        <v>46028.907905092594</v>
+        <v>46065.655185185184</v>
       </c>
       <c r="E57" s="8">
-        <v>46028.907905092594</v>
+        <v>46065.655185185184</v>
       </c>
       <c r="F57" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G57" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H57" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I57" s="7">
-        <v>1394721</v>
+        <v>1411990</v>
       </c>
       <c r="J57" s="5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="K57" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="L57" s="7" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="M57" s="10"/>
       <c r="N57" s="10">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="O57" s="7"/>
     </row>
     <row r="58" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A58" s="2"/>
       <c r="B58" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C58" s="7" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="8">
-        <v>46029.6719212963</v>
+        <v>46066.613657407404</v>
       </c>
       <c r="E58" s="8">
-        <v>46029.6719212963</v>
+        <v>46066.613657407404</v>
       </c>
       <c r="F58" s="7" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G58" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H58" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I58" s="7">
-        <v>1394721</v>
+        <v>1411990</v>
       </c>
       <c r="J58" s="5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="K58" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="L58" s="7" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="M58" s="10"/>
       <c r="N58" s="10">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O58" s="7"/>
     </row>
     <row r="59" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A59" s="2"/>
       <c r="B59" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D59" s="8">
-        <v>46034.72855324074</v>
+        <v>46066.670127314814</v>
       </c>
       <c r="E59" s="8">
-        <v>46034.72855324074</v>
+        <v>46066.670127314814</v>
       </c>
       <c r="F59" s="7" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G59" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H59" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I59" s="7">
-        <v>1394721</v>
+        <v>1411990</v>
       </c>
       <c r="J59" s="5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="K59" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="L59" s="7" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="M59" s="10"/>
       <c r="N59" s="10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O59" s="7"/>
     </row>
@@ -3277,38 +3280,38 @@
         <v>5</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="D60" s="8">
-        <v>46037.838958333334</v>
+        <v>46028.907905092594</v>
       </c>
       <c r="E60" s="8">
-        <v>46037.838958333334</v>
+        <v>46028.907905092594</v>
       </c>
       <c r="F60" s="7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G60" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H60" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I60" s="7">
         <v>1394721</v>
       </c>
       <c r="J60" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K60" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L60" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M60" s="10"/>
       <c r="N60" s="10">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="O60" s="7"/>
     </row>
@@ -3318,38 +3321,38 @@
         <v>5</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D61" s="8">
-        <v>46042.727754629632</v>
+        <v>46029.6719212963</v>
       </c>
       <c r="E61" s="8">
-        <v>46042.727754629632</v>
+        <v>46029.6719212963</v>
       </c>
       <c r="F61" s="7" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G61" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H61" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I61" s="7">
         <v>1394721</v>
       </c>
       <c r="J61" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K61" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L61" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M61" s="10"/>
       <c r="N61" s="10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O61" s="7"/>
     </row>
@@ -3359,38 +3362,38 @@
         <v>5</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="D62" s="8">
-        <v>46043.627881944441</v>
+        <v>46034.72855324074</v>
       </c>
       <c r="E62" s="8">
-        <v>46043.627881944441</v>
+        <v>46034.72855324074</v>
       </c>
       <c r="F62" s="7" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="G62" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H62" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I62" s="7">
-        <v>1410339</v>
+        <v>1394721</v>
       </c>
       <c r="J62" s="5" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="K62" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L62" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M62" s="10"/>
       <c r="N62" s="10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O62" s="7"/>
     </row>
@@ -3400,38 +3403,38 @@
         <v>5</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D63" s="8">
-        <v>46052.626018518517</v>
+        <v>46037.838958333334</v>
       </c>
       <c r="E63" s="8">
-        <v>46052.626018518517</v>
+        <v>46037.838958333334</v>
       </c>
       <c r="F63" s="7" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="G63" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H63" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I63" s="7">
-        <v>1411706</v>
+        <v>1394721</v>
       </c>
       <c r="J63" s="5" t="s">
         <v>76</v>
       </c>
       <c r="K63" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L63" s="7" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="M63" s="10"/>
       <c r="N63" s="10">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="O63" s="7"/>
     </row>
@@ -3441,38 +3444,38 @@
         <v>5</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="D64" s="8">
-        <v>46053.632291666669</v>
+        <v>46042.727754629632</v>
       </c>
       <c r="E64" s="8">
-        <v>46053.632291666669</v>
+        <v>46042.727754629632</v>
       </c>
       <c r="F64" s="7" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="G64" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H64" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I64" s="7">
-        <v>1411708</v>
+        <v>1394721</v>
       </c>
       <c r="J64" s="5" t="s">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="K64" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L64" s="7" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="M64" s="10"/>
       <c r="N64" s="10">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="O64" s="7"/>
     </row>
@@ -3482,34 +3485,34 @@
         <v>5</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="D65" s="8">
-        <v>46071.601446759261</v>
+        <v>46043.627881944441</v>
       </c>
       <c r="E65" s="8">
-        <v>46071.601446759261</v>
+        <v>46043.627881944441</v>
       </c>
       <c r="F65" s="7" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G65" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H65" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I65" s="7">
-        <v>1418251</v>
+        <v>1410339</v>
       </c>
       <c r="J65" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="K65" s="5" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="L65" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M65" s="10"/>
       <c r="N65" s="10">
@@ -3523,198 +3526,198 @@
         <v>5</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D66" s="8">
-        <v>46076.679282407407</v>
+        <v>46052.626018518517</v>
       </c>
       <c r="E66" s="8">
-        <v>46076.679282407407</v>
+        <v>46052.626018518517</v>
       </c>
       <c r="F66" s="7" t="s">
         <v>55</v>
       </c>
       <c r="G66" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H66" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I66" s="7">
-        <v>1422511</v>
+        <v>1411706</v>
       </c>
       <c r="J66" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="K66" s="5" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="L66" s="7" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="M66" s="10"/>
       <c r="N66" s="10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O66" s="7"/>
     </row>
     <row r="67" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A67" s="2"/>
       <c r="B67" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="D67" s="8">
-        <v>46027.633611111109</v>
+        <v>46053.632291666669</v>
       </c>
       <c r="E67" s="8">
-        <v>46027.633611111109</v>
+        <v>46053.632291666669</v>
       </c>
       <c r="F67" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G67" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H67" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I67" s="7">
-        <v>1404289</v>
+        <v>1411708</v>
       </c>
       <c r="J67" s="5" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K67" s="5" t="s">
         <v>99</v>
       </c>
       <c r="L67" s="7" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="M67" s="10"/>
       <c r="N67" s="10">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="O67" s="7"/>
     </row>
     <row r="68" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A68" s="2"/>
       <c r="B68" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="D68" s="8">
-        <v>46029.802372685182</v>
+        <v>46071.601446759261</v>
       </c>
       <c r="E68" s="8">
-        <v>46029.802372685182</v>
+        <v>46071.601446759261</v>
       </c>
       <c r="F68" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G68" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H68" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I68" s="7">
-        <v>1394724</v>
+        <v>1418251</v>
       </c>
       <c r="J68" s="5" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="K68" s="5" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="L68" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M68" s="10"/>
       <c r="N68" s="10">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O68" s="7"/>
     </row>
     <row r="69" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A69" s="2"/>
       <c r="B69" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="D69" s="8">
-        <v>46030.908472222225</v>
+        <v>46076.679282407407</v>
       </c>
       <c r="E69" s="8">
-        <v>46030.908472222225</v>
+        <v>46076.679282407407</v>
       </c>
       <c r="F69" s="7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G69" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H69" s="5" t="s">
         <v>67</v>
       </c>
       <c r="I69" s="7">
-        <v>1394724</v>
+        <v>1422511</v>
       </c>
       <c r="J69" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="K69" s="5" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="L69" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M69" s="10"/>
       <c r="N69" s="10">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O69" s="7"/>
     </row>
     <row r="70" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A70" s="2"/>
       <c r="B70" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="D70" s="8">
-        <v>46031.590057870373</v>
+        <v>46077.591944444444</v>
       </c>
       <c r="E70" s="8">
-        <v>46031.590057870373</v>
+        <v>46077.591944444444</v>
       </c>
       <c r="F70" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G70" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H70" s="5" t="s">
         <v>67</v>
       </c>
       <c r="I70" s="7">
-        <v>1394724</v>
+        <v>1422511</v>
       </c>
       <c r="J70" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="K70" s="5" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="L70" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M70" s="10"/>
       <c r="N70" s="10">
@@ -3725,160 +3728,160 @@
     <row r="71" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A71" s="2"/>
       <c r="B71" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="D71" s="8">
-        <v>46076.8827662037</v>
+        <v>46077.861296296294</v>
       </c>
       <c r="E71" s="8">
-        <v>46076.8827662037</v>
+        <v>46077.861296296294</v>
       </c>
       <c r="F71" s="7" t="s">
         <v>57</v>
       </c>
       <c r="G71" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H71" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I71" s="7">
-        <v>1422286</v>
+        <v>1422511</v>
       </c>
       <c r="J71" s="5" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="K71" s="5" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="L71" s="7" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="M71" s="10"/>
       <c r="N71" s="10">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="O71" s="7"/>
     </row>
     <row r="72" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A72" s="2"/>
       <c r="B72" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D72" s="8">
-        <v>46024.795127314814</v>
+        <v>46027.633611111109</v>
       </c>
       <c r="E72" s="8">
-        <v>46024.795127314814</v>
+        <v>46027.633611111109</v>
       </c>
       <c r="F72" s="7" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="G72" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H72" s="5" t="s">
         <v>67</v>
       </c>
       <c r="I72" s="7">
-        <v>1398335</v>
+        <v>1404289</v>
       </c>
       <c r="J72" s="5" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="K72" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L72" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M72" s="10"/>
       <c r="N72" s="10">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="O72" s="7"/>
     </row>
     <row r="73" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A73" s="2"/>
       <c r="B73" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C73" s="7" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="D73" s="8">
-        <v>46024.795277777775</v>
+        <v>46029.802372685182</v>
       </c>
       <c r="E73" s="8">
-        <v>46024.795277777775</v>
+        <v>46029.802372685182</v>
       </c>
       <c r="F73" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G73" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H73" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I73" s="7">
-        <v>1398335</v>
+        <v>1394724</v>
       </c>
       <c r="J73" s="5" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="K73" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L73" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M73" s="10"/>
       <c r="N73" s="10">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="O73" s="7"/>
     </row>
     <row r="74" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A74" s="2"/>
       <c r="B74" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C74" s="7" t="s">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="D74" s="8">
-        <v>46024.900324074071</v>
+        <v>46030.908472222225</v>
       </c>
       <c r="E74" s="8">
-        <v>46024.900324074071</v>
+        <v>46030.908472222225</v>
       </c>
       <c r="F74" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G74" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H74" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I74" s="7">
-        <v>1398335</v>
+        <v>1394724</v>
       </c>
       <c r="J74" s="5" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="K74" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L74" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M74" s="10"/>
       <c r="N74" s="10">
@@ -3889,82 +3892,82 @@
     <row r="75" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A75" s="2"/>
       <c r="B75" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C75" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D75" s="8">
-        <v>46028.866898148146</v>
+        <v>46031.590057870373</v>
       </c>
       <c r="E75" s="8">
-        <v>46028.866898148146</v>
+        <v>46031.590057870373</v>
       </c>
       <c r="F75" s="7" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G75" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H75" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I75" s="7">
-        <v>1402956</v>
+        <v>1394724</v>
       </c>
       <c r="J75" s="5" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="K75" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L75" s="7" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="M75" s="10"/>
       <c r="N75" s="10">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O75" s="7"/>
     </row>
     <row r="76" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A76" s="2"/>
       <c r="B76" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C76" s="7" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D76" s="8">
-        <v>46034.751261574071</v>
+        <v>46076.8827662037</v>
       </c>
       <c r="E76" s="8">
-        <v>46034.751261574071</v>
+        <v>46076.8827662037</v>
       </c>
       <c r="F76" s="7" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="G76" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H76" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I76" s="7">
-        <v>1404958</v>
+        <v>1422286</v>
       </c>
       <c r="J76" s="5" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="K76" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L76" s="7" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="M76" s="10"/>
       <c r="N76" s="10">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="O76" s="7"/>
     </row>
@@ -3974,38 +3977,38 @@
         <v>7</v>
       </c>
       <c r="C77" s="7" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="D77" s="8">
-        <v>46062.904895833337</v>
+        <v>46024.795127314814</v>
       </c>
       <c r="E77" s="8">
-        <v>46062.904895833337</v>
+        <v>46024.795127314814</v>
       </c>
       <c r="F77" s="7" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="G77" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H77" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I77" s="7">
-        <v>1412987</v>
+        <v>1398335</v>
       </c>
       <c r="J77" s="5" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="K77" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L77" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M77" s="10"/>
       <c r="N77" s="10">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="O77" s="7"/>
     </row>
@@ -4018,35 +4021,35 @@
         <v>42</v>
       </c>
       <c r="D78" s="8">
-        <v>46063.874467592592</v>
+        <v>46024.795277777775</v>
       </c>
       <c r="E78" s="8">
-        <v>46063.874467592592</v>
+        <v>46024.795277777775</v>
       </c>
       <c r="F78" s="7" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="G78" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H78" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I78" s="7">
-        <v>1412987</v>
+        <v>1398335</v>
       </c>
       <c r="J78" s="5" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="K78" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L78" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M78" s="10"/>
       <c r="N78" s="10">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O78" s="7"/>
     </row>
@@ -4056,38 +4059,38 @@
         <v>7</v>
       </c>
       <c r="C79" s="7" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D79" s="8">
-        <v>46067.906875000001</v>
+        <v>46024.900324074071</v>
       </c>
       <c r="E79" s="8">
-        <v>46067.906875000001</v>
+        <v>46024.900324074071</v>
       </c>
       <c r="F79" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G79" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H79" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I79" s="7">
-        <v>1411991</v>
+        <v>1398335</v>
       </c>
       <c r="J79" s="5" t="s">
         <v>94</v>
       </c>
       <c r="K79" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L79" s="7" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="M79" s="10"/>
       <c r="N79" s="10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O79" s="7"/>
     </row>
@@ -4097,87 +4100,333 @@
         <v>7</v>
       </c>
       <c r="C80" s="7" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="D80" s="8">
-        <v>46069.700543981482</v>
+        <v>46028.866898148146</v>
       </c>
       <c r="E80" s="8">
-        <v>46069.700543981482</v>
+        <v>46028.866898148146</v>
       </c>
       <c r="F80" s="7" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="G80" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H80" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I80" s="7">
-        <v>1411991</v>
+        <v>1402956</v>
       </c>
       <c r="J80" s="5" t="s">
-        <v>94</v>
+        <v>77</v>
       </c>
       <c r="K80" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L80" s="7" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="M80" s="10"/>
       <c r="N80" s="10">
+        <v>2</v>
+      </c>
+      <c r="O80" s="7"/>
+    </row>
+    <row r="81" spans="1:15" ht="21" x14ac:dyDescent="0.2">
+      <c r="A81" s="2"/>
+      <c r="B81" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C81" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D81" s="8">
+        <v>46034.751261574071</v>
+      </c>
+      <c r="E81" s="8">
+        <v>46034.751261574071</v>
+      </c>
+      <c r="F81" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="G81" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="H81" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="I81" s="7">
+        <v>1404958</v>
+      </c>
+      <c r="J81" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="K81" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="L81" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="M81" s="10"/>
+      <c r="N81" s="10">
+        <v>7</v>
+      </c>
+      <c r="O81" s="7"/>
+    </row>
+    <row r="82" spans="1:15" ht="21" x14ac:dyDescent="0.2">
+      <c r="A82" s="2"/>
+      <c r="B82" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C82" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D82" s="8">
+        <v>46062.904895833337</v>
+      </c>
+      <c r="E82" s="8">
+        <v>46062.904895833337</v>
+      </c>
+      <c r="F82" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="G82" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="H82" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="I82" s="7">
+        <v>1412987</v>
+      </c>
+      <c r="J82" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="K82" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="L82" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="M82" s="10"/>
+      <c r="N82" s="10">
+        <v>1</v>
+      </c>
+      <c r="O82" s="7"/>
+    </row>
+    <row r="83" spans="1:15" ht="21" x14ac:dyDescent="0.2">
+      <c r="A83" s="2"/>
+      <c r="B83" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C83" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D83" s="8">
+        <v>46063.874467592592</v>
+      </c>
+      <c r="E83" s="8">
+        <v>46063.874467592592</v>
+      </c>
+      <c r="F83" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="G83" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="H83" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="I83" s="7">
+        <v>1412987</v>
+      </c>
+      <c r="J83" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="K83" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="L83" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="M83" s="10"/>
+      <c r="N83" s="10">
+        <v>5</v>
+      </c>
+      <c r="O83" s="7"/>
+    </row>
+    <row r="84" spans="1:15" ht="21" x14ac:dyDescent="0.2">
+      <c r="A84" s="2"/>
+      <c r="B84" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C84" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D84" s="8">
+        <v>46067.906875000001</v>
+      </c>
+      <c r="E84" s="8">
+        <v>46067.906875000001</v>
+      </c>
+      <c r="F84" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="G84" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="H84" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="I84" s="7">
+        <v>1411991</v>
+      </c>
+      <c r="J84" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="K84" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="L84" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="M84" s="10"/>
+      <c r="N84" s="10">
+        <v>3</v>
+      </c>
+      <c r="O84" s="7"/>
+    </row>
+    <row r="85" spans="1:15" ht="21" x14ac:dyDescent="0.2">
+      <c r="A85" s="2"/>
+      <c r="B85" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C85" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D85" s="8">
+        <v>46069.700543981482</v>
+      </c>
+      <c r="E85" s="8">
+        <v>46069.700543981482</v>
+      </c>
+      <c r="F85" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="G85" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="H85" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="I85" s="7">
+        <v>1411991</v>
+      </c>
+      <c r="J85" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="K85" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="L85" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="M85" s="10"/>
+      <c r="N85" s="10">
         <v>10</v>
       </c>
-      <c r="O80" s="7"/>
-    </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A81" s="4"/>
-      <c r="B81" s="6"/>
-      <c r="C81" s="6"/>
-      <c r="D81" s="6"/>
-      <c r="E81" s="6"/>
-      <c r="F81" s="6"/>
-      <c r="G81" s="6"/>
-      <c r="H81" s="6"/>
-      <c r="I81" s="6"/>
-      <c r="J81" s="6"/>
-      <c r="K81" s="6"/>
-      <c r="L81" s="6"/>
-      <c r="M81" s="9">
+      <c r="O85" s="7"/>
+    </row>
+    <row r="86" spans="1:15" ht="21" x14ac:dyDescent="0.2">
+      <c r="A86" s="2"/>
+      <c r="B86" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C86" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D86" s="8">
+        <v>46077.65824074074</v>
+      </c>
+      <c r="E86" s="8">
+        <v>46077.65824074074</v>
+      </c>
+      <c r="F86" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="G86" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="H86" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="I86" s="7">
+        <v>1422285</v>
+      </c>
+      <c r="J86" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="K86" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="L86" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="M86" s="10"/>
+      <c r="N86" s="10">
+        <v>1</v>
+      </c>
+      <c r="O86" s="7"/>
+    </row>
+    <row r="87" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A87" s="4"/>
+      <c r="B87" s="6"/>
+      <c r="C87" s="6"/>
+      <c r="D87" s="6"/>
+      <c r="E87" s="6"/>
+      <c r="F87" s="6"/>
+      <c r="G87" s="6"/>
+      <c r="H87" s="6"/>
+      <c r="I87" s="6"/>
+      <c r="J87" s="6"/>
+      <c r="K87" s="6"/>
+      <c r="L87" s="6"/>
+      <c r="M87" s="9">
         <v>0</v>
       </c>
-      <c r="N81" s="9">
-        <v>160</v>
-      </c>
-      <c r="O81" s="9">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A82" s="4"/>
-      <c r="B82" s="6"/>
-      <c r="C82" s="6"/>
-      <c r="D82" s="6"/>
-      <c r="E82" s="6"/>
-      <c r="F82" s="6"/>
-      <c r="G82" s="6"/>
-      <c r="H82" s="9">
-        <v>75</v>
-      </c>
-      <c r="I82" s="6"/>
-      <c r="J82" s="6"/>
-      <c r="K82" s="6"/>
-      <c r="L82" s="6"/>
-      <c r="M82" s="9">
+      <c r="N87" s="9">
+        <v>177</v>
+      </c>
+      <c r="O87" s="9">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="88" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A88" s="4"/>
+      <c r="B88" s="6"/>
+      <c r="C88" s="6"/>
+      <c r="D88" s="6"/>
+      <c r="E88" s="6"/>
+      <c r="F88" s="6"/>
+      <c r="G88" s="6"/>
+      <c r="H88" s="9">
+        <v>81</v>
+      </c>
+      <c r="I88" s="6"/>
+      <c r="J88" s="6"/>
+      <c r="K88" s="6"/>
+      <c r="L88" s="6"/>
+      <c r="M88" s="9">
         <v>0</v>
       </c>
-      <c r="N82" s="9">
-        <v>355</v>
-      </c>
-      <c r="O82" s="9">
-        <v>75</v>
+      <c r="N88" s="9">
+        <v>380</v>
+      </c>
+      <c r="O88" s="9">
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -4187,8 +4436,9 @@
     <mergeCell ref="M1:O1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="B3:O3"/>
-    <mergeCell ref="B48:O48"/>
+    <mergeCell ref="B51:O51"/>
   </mergeCells>
   <pageMargins left="0.78740157499999996" right="0.78740157499999996" top="0.984251969" bottom="0.984251969" header="0.4921259845" footer="0.4921259845"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica (28/02/2026  8:15:07,69)
</commit_message>
<xml_diff>
--- a/rejeito.xlsx
+++ b/rejeito.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PLANILHAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AD2107F8-81A5-4303-A254-36AF54E01960}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E7B0AA9F-BDD3-4DB8-AEBB-E50A9FEA6FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3930" yWindow="3930" windowWidth="21600" windowHeight="11295" xr2:uid="{8EC2283C-B3A0-459D-A031-B95FA7985C31}"/>
+    <workbookView xWindow="3585" yWindow="3585" windowWidth="21600" windowHeight="11295" xr2:uid="{4F01A82A-6053-40A1-B740-48809F7DEDF6}"/>
   </bookViews>
   <sheets>
     <sheet name="rejeito" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="717" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="757" uniqueCount="118">
   <si>
     <t>Dados</t>
   </si>
@@ -112,6 +112,9 @@
     <t>16/02/2026</t>
   </si>
   <si>
+    <t>27/02/2026</t>
+  </si>
+  <si>
     <t>22/01/2026</t>
   </si>
   <si>
@@ -283,13 +286,13 @@
     <t xml:space="preserve">CI003141-EM-CASA-961 - COPO CAFÉ FACETADO C/ IMPRESSÃO DIGITAL </t>
   </si>
   <si>
+    <t xml:space="preserve">CI003141-EM-CASA-1388 - COPO CAFÉ FACETADO C/ IMPRESSÃO DIGITAL </t>
+  </si>
+  <si>
     <t>CIPF002816STITCHCAP2624 - CORPO GARRAFA FUN 600 ML - STITCH CAPIVA</t>
   </si>
   <si>
     <t>CIPF002816-PRINCESAS-24 - CORPO GARRAFA FUN 600 ML - PRINCESAS 202</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CI003141-EM-CASA-1388 - COPO CAFÉ FACETADO C/ IMPRESSÃO DIGITAL </t>
   </si>
   <si>
     <t xml:space="preserve">CI002027-ARIEL_23-24 - CORPO GARRAFA RETRÔ 500ML SOPRO - ARIEL </t>
@@ -915,8 +918,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{987863C2-E270-4F1A-9430-C8823FDC7009}">
-  <dimension ref="A1:O94"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24E902DF-2118-4D25-BEFA-B7AF8A662001}">
+  <dimension ref="A1:O99"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.42578125" customWidth="1"/>
@@ -947,14 +950,14 @@
       <c r="F1" s="11"/>
       <c r="G1" s="11"/>
       <c r="H1" s="11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I1" s="11"/>
       <c r="J1" s="11"/>
       <c r="K1" s="11"/>
       <c r="L1" s="11"/>
       <c r="M1" s="11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="N1" s="11"/>
       <c r="O1" s="11"/>
@@ -968,40 +971,40 @@
         <v>9</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3" spans="1:15" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1040,25 +1043,25 @@
         <v>46046.443344907406</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I4" s="7">
         <v>1406207</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M4" s="10"/>
       <c r="N4" s="10">
@@ -1081,25 +1084,25 @@
         <v>46046.553217592591</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I5" s="7">
         <v>1406207</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M5" s="10"/>
       <c r="N5" s="10">
@@ -1122,25 +1125,25 @@
         <v>46050.493333333332</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I6" s="7">
         <v>1411349</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L6" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="M6" s="10"/>
       <c r="N6" s="10">
@@ -1163,25 +1166,25 @@
         <v>46051.555428240739</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I7" s="7">
         <v>1411348</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="M7" s="10"/>
       <c r="N7" s="10">
@@ -1204,25 +1207,25 @@
         <v>46053.377129629633</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I8" s="7">
         <v>1409954</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M8" s="10"/>
       <c r="N8" s="10">
@@ -1245,25 +1248,25 @@
         <v>46062.302418981482</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I9" s="7">
         <v>1411984</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L9" s="7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="M9" s="10"/>
       <c r="N9" s="10">
@@ -1286,25 +1289,25 @@
         <v>46062.570879629631</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I10" s="7">
         <v>1411984</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="M10" s="10"/>
       <c r="N10" s="10">
@@ -1327,25 +1330,25 @@
         <v>46064.297777777778</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I11" s="7">
         <v>1411984</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L11" s="7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="M11" s="10"/>
       <c r="N11" s="10">
@@ -1368,25 +1371,25 @@
         <v>46064.455104166664</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I12" s="7">
         <v>1411990</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="M12" s="10"/>
       <c r="N12" s="10">
@@ -1409,25 +1412,25 @@
         <v>46028.331469907411</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I13" s="7">
         <v>1402958</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L13" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M13" s="10"/>
       <c r="N13" s="10">
@@ -1450,25 +1453,25 @@
         <v>46030.306192129632</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I14" s="7">
         <v>1394721</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L14" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M14" s="10"/>
       <c r="N14" s="10">
@@ -1491,25 +1494,25 @@
         <v>46031.443101851852</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I15" s="7">
         <v>1394721</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M15" s="10"/>
       <c r="N15" s="10">
@@ -1532,25 +1535,25 @@
         <v>46035.530381944445</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I16" s="7">
         <v>1394721</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L16" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M16" s="10"/>
       <c r="N16" s="10">
@@ -1573,25 +1576,25 @@
         <v>46046.391701388886</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I17" s="7">
         <v>1410340</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L17" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M17" s="10"/>
       <c r="N17" s="10">
@@ -1614,25 +1617,25 @@
         <v>46046.516597222224</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I18" s="7">
         <v>1410340</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L18" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M18" s="10"/>
       <c r="N18" s="10">
@@ -1655,25 +1658,25 @@
         <v>46048.278912037036</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I19" s="7">
         <v>1410340</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K19" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L19" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M19" s="10"/>
       <c r="N19" s="10">
@@ -1696,25 +1699,25 @@
         <v>46051.403391203705</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I20" s="7">
         <v>1410340</v>
       </c>
       <c r="J20" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K20" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L20" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M20" s="10"/>
       <c r="N20" s="10">
@@ -1737,25 +1740,25 @@
         <v>46053.550381944442</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I21" s="7">
         <v>1411706</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L21" s="7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="M21" s="10"/>
       <c r="N21" s="10">
@@ -1778,25 +1781,25 @@
         <v>46057.413171296299</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I22" s="7">
         <v>1411704</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L22" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M22" s="10"/>
       <c r="N22" s="10">
@@ -1819,25 +1822,25 @@
         <v>46058.357476851852</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I23" s="7">
         <v>1411704</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L23" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M23" s="10"/>
       <c r="N23" s="10">
@@ -1860,25 +1863,25 @@
         <v>46058.531793981485</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I24" s="7">
         <v>1411704</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L24" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M24" s="10"/>
       <c r="N24" s="10">
@@ -1901,25 +1904,25 @@
         <v>46067.433020833334</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I25" s="7">
         <v>1418256</v>
       </c>
       <c r="J25" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L25" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M25" s="10"/>
       <c r="N25" s="10">
@@ -1942,25 +1945,25 @@
         <v>46073.579664351855</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I26" s="7">
         <v>1422511</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L26" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M26" s="10"/>
       <c r="N26" s="10">
@@ -1983,25 +1986,25 @@
         <v>46077.38318287037</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I27" s="7">
         <v>1422511</v>
       </c>
       <c r="J27" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L27" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M27" s="10"/>
       <c r="N27" s="10">
@@ -2024,25 +2027,25 @@
         <v>46078.372766203705</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I28" s="7">
         <v>1422511</v>
       </c>
       <c r="J28" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L28" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M28" s="10"/>
       <c r="N28" s="10">
@@ -2065,25 +2068,25 @@
         <v>46027.4840625</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I29" s="7">
         <v>1404289</v>
       </c>
       <c r="J29" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L29" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M29" s="10"/>
       <c r="N29" s="10">
@@ -2106,25 +2109,25 @@
         <v>46030.397997685184</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G30" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I30" s="7">
         <v>1394724</v>
       </c>
       <c r="J30" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L30" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M30" s="10"/>
       <c r="N30" s="10">
@@ -2147,25 +2150,25 @@
         <v>46030.408148148148</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G31" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I31" s="7">
         <v>1394724</v>
       </c>
       <c r="J31" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L31" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M31" s="10"/>
       <c r="N31" s="10">
@@ -2188,25 +2191,25 @@
         <v>46030.478854166664</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G32" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I32" s="7">
         <v>1394724</v>
       </c>
       <c r="J32" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L32" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M32" s="10"/>
       <c r="N32" s="10">
@@ -2229,25 +2232,25 @@
         <v>46030.561284722222</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G33" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I33" s="7">
         <v>1394724</v>
       </c>
       <c r="J33" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L33" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M33" s="10"/>
       <c r="N33" s="10">
@@ -2270,25 +2273,25 @@
         <v>46035.478368055556</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G34" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I34" s="7">
         <v>1394724</v>
       </c>
       <c r="J34" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L34" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M34" s="10"/>
       <c r="N34" s="10">
@@ -2311,25 +2314,25 @@
         <v>46043.385474537034</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G35" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I35" s="7">
         <v>1394724</v>
       </c>
       <c r="J35" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K35" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L35" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M35" s="10"/>
       <c r="N35" s="10">
@@ -2352,25 +2355,25 @@
         <v>46043.565196759257</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G36" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H36" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I36" s="7">
         <v>1394724</v>
       </c>
       <c r="J36" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L36" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M36" s="10"/>
       <c r="N36" s="10">
@@ -2393,25 +2396,25 @@
         <v>46069.559953703705</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G37" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H37" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I37" s="7">
         <v>1421099</v>
       </c>
       <c r="J37" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L37" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M37" s="10"/>
       <c r="N37" s="10">
@@ -2434,25 +2437,25 @@
         <v>46078.552407407406</v>
       </c>
       <c r="F38" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G38" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H38" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I38" s="7">
         <v>1422286</v>
       </c>
       <c r="J38" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L38" s="7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="M38" s="10"/>
       <c r="N38" s="10">
@@ -2463,82 +2466,82 @@
     <row r="39" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A39" s="2"/>
       <c r="B39" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="D39" s="8">
-        <v>46035.47824074074</v>
+        <v>46080.522418981483</v>
       </c>
       <c r="E39" s="8">
-        <v>46035.47824074074</v>
+        <v>46080.522418981483</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G39" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I39" s="7">
-        <v>1404958</v>
+        <v>1422285</v>
       </c>
       <c r="J39" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="K39" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L39" s="7" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="M39" s="10"/>
       <c r="N39" s="10">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="O39" s="7"/>
     </row>
     <row r="40" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A40" s="2"/>
       <c r="B40" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D40" s="8">
-        <v>46043.385196759256</v>
+        <v>46080.532164351855</v>
       </c>
       <c r="E40" s="8">
-        <v>46043.385196759256</v>
+        <v>46080.532164351855</v>
       </c>
       <c r="F40" s="7" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G40" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H40" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I40" s="7">
-        <v>1405794</v>
+        <v>1422285</v>
       </c>
       <c r="J40" s="5" t="s">
         <v>88</v>
       </c>
       <c r="K40" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L40" s="7" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="M40" s="10"/>
       <c r="N40" s="10">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="O40" s="7"/>
     </row>
@@ -2548,38 +2551,38 @@
         <v>7</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="D41" s="8">
-        <v>46043.385289351849</v>
+        <v>46035.47824074074</v>
       </c>
       <c r="E41" s="8">
-        <v>46043.385289351849</v>
+        <v>46035.47824074074</v>
       </c>
       <c r="F41" s="7" t="s">
         <v>52</v>
       </c>
       <c r="G41" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H41" s="5" t="s">
         <v>70</v>
       </c>
       <c r="I41" s="7">
-        <v>1405794</v>
+        <v>1404958</v>
       </c>
       <c r="J41" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K41" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L41" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M41" s="10"/>
       <c r="N41" s="10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O41" s="7"/>
     </row>
@@ -2592,35 +2595,35 @@
         <v>28</v>
       </c>
       <c r="D42" s="8">
-        <v>46043.441296296296</v>
+        <v>46043.385196759256</v>
       </c>
       <c r="E42" s="8">
-        <v>46043.441296296296</v>
+        <v>46043.385196759256</v>
       </c>
       <c r="F42" s="7" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G42" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H42" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I42" s="7">
         <v>1405794</v>
       </c>
       <c r="J42" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="K42" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L42" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M42" s="10"/>
       <c r="N42" s="10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O42" s="7"/>
     </row>
@@ -2630,34 +2633,34 @@
         <v>7</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D43" s="8">
-        <v>46044.570300925923</v>
+        <v>46043.385289351849</v>
       </c>
       <c r="E43" s="8">
-        <v>46044.570300925923</v>
+        <v>46043.385289351849</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="G43" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H43" s="5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I43" s="7">
         <v>1405794</v>
       </c>
       <c r="J43" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="K43" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L43" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M43" s="10"/>
       <c r="N43" s="10">
@@ -2671,38 +2674,38 @@
         <v>7</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="D44" s="8">
-        <v>46050.574884259258</v>
+        <v>46043.441296296296</v>
       </c>
       <c r="E44" s="8">
-        <v>46050.574884259258</v>
+        <v>46043.441296296296</v>
       </c>
       <c r="F44" s="7" t="s">
         <v>50</v>
       </c>
       <c r="G44" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H44" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I44" s="7">
-        <v>1411351</v>
+        <v>1405794</v>
       </c>
       <c r="J44" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K44" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L44" s="7" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="M44" s="10"/>
       <c r="N44" s="10">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="O44" s="7"/>
     </row>
@@ -2712,38 +2715,38 @@
         <v>7</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="D45" s="8">
-        <v>46051.280300925922</v>
+        <v>46044.570300925923</v>
       </c>
       <c r="E45" s="8">
-        <v>46051.280300925922</v>
+        <v>46044.570300925923</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="G45" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H45" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I45" s="7">
-        <v>1411352</v>
+        <v>1405794</v>
       </c>
       <c r="J45" s="5" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="K45" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L45" s="7" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="M45" s="10"/>
       <c r="N45" s="10">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O45" s="7"/>
     </row>
@@ -2753,38 +2756,38 @@
         <v>7</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="D46" s="8">
-        <v>46056.33489583333</v>
+        <v>46050.574884259258</v>
       </c>
       <c r="E46" s="8">
-        <v>46056.33489583333</v>
+        <v>46050.574884259258</v>
       </c>
       <c r="F46" s="7" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="G46" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H46" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I46" s="7">
-        <v>1410338</v>
+        <v>1411351</v>
       </c>
       <c r="J46" s="5" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="K46" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L46" s="7" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="M46" s="10"/>
       <c r="N46" s="10">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="O46" s="7"/>
     </row>
@@ -2794,38 +2797,38 @@
         <v>7</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D47" s="8">
-        <v>46062.345243055555</v>
+        <v>46051.280300925922</v>
       </c>
       <c r="E47" s="8">
-        <v>46062.345243055555</v>
+        <v>46051.280300925922</v>
       </c>
       <c r="F47" s="7" t="s">
         <v>56</v>
       </c>
       <c r="G47" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H47" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I47" s="7">
-        <v>1412987</v>
+        <v>1411352</v>
       </c>
       <c r="J47" s="5" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="K47" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L47" s="7" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="M47" s="10"/>
       <c r="N47" s="10">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O47" s="7"/>
     </row>
@@ -2835,38 +2838,38 @@
         <v>7</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="D48" s="8">
-        <v>46064.292500000003</v>
+        <v>46056.33489583333</v>
       </c>
       <c r="E48" s="8">
-        <v>46064.292500000003</v>
+        <v>46056.33489583333</v>
       </c>
       <c r="F48" s="7" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G48" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H48" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I48" s="7">
-        <v>1412987</v>
+        <v>1410338</v>
       </c>
       <c r="J48" s="5" t="s">
         <v>91</v>
       </c>
       <c r="K48" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L48" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M48" s="10"/>
       <c r="N48" s="10">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="O48" s="7"/>
     </row>
@@ -2876,38 +2879,38 @@
         <v>7</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D49" s="8">
-        <v>46073.402627314812</v>
+        <v>46062.345243055555</v>
       </c>
       <c r="E49" s="8">
-        <v>46073.402627314812</v>
+        <v>46062.345243055555</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="G49" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H49" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I49" s="7">
-        <v>1421099</v>
+        <v>1412987</v>
       </c>
       <c r="J49" s="5" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="K49" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L49" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M49" s="10"/>
       <c r="N49" s="10">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="O49" s="7"/>
     </row>
@@ -2917,34 +2920,34 @@
         <v>7</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D50" s="8">
-        <v>46077.368379629632</v>
+        <v>46064.292500000003</v>
       </c>
       <c r="E50" s="8">
-        <v>46077.368379629632</v>
+        <v>46064.292500000003</v>
       </c>
       <c r="F50" s="7" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G50" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H50" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I50" s="7">
-        <v>1422285</v>
+        <v>1412987</v>
       </c>
       <c r="J50" s="5" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="K50" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L50" s="7" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="M50" s="10"/>
       <c r="N50" s="10">
@@ -2958,166 +2961,166 @@
         <v>7</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D51" s="8">
-        <v>46077.554594907408</v>
+        <v>46073.402627314812</v>
       </c>
       <c r="E51" s="8">
-        <v>46077.554594907408</v>
+        <v>46073.402627314812</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="G51" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H51" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I51" s="7">
-        <v>1422285</v>
+        <v>1421099</v>
       </c>
       <c r="J51" s="5" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="K51" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L51" s="7" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="M51" s="10"/>
       <c r="N51" s="10">
+        <v>2</v>
+      </c>
+      <c r="O51" s="7"/>
+    </row>
+    <row r="52" spans="1:15" ht="21" x14ac:dyDescent="0.2">
+      <c r="A52" s="2"/>
+      <c r="B52" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C52" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D52" s="8">
+        <v>46077.368379629632</v>
+      </c>
+      <c r="E52" s="8">
+        <v>46077.368379629632</v>
+      </c>
+      <c r="F52" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="G52" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="H52" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="I52" s="7">
+        <v>1422285</v>
+      </c>
+      <c r="J52" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="K52" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="L52" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="M52" s="10"/>
+      <c r="N52" s="10">
         <v>3</v>
       </c>
-      <c r="O51" s="7"/>
-    </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A52" s="4"/>
-      <c r="B52" s="6"/>
-      <c r="C52" s="6"/>
-      <c r="D52" s="6"/>
-      <c r="E52" s="6"/>
-      <c r="F52" s="6"/>
-      <c r="G52" s="6"/>
-      <c r="H52" s="6"/>
-      <c r="I52" s="6"/>
-      <c r="J52" s="6"/>
-      <c r="K52" s="6"/>
-      <c r="L52" s="6"/>
-      <c r="M52" s="9">
+      <c r="O52" s="7"/>
+    </row>
+    <row r="53" spans="1:15" ht="21" x14ac:dyDescent="0.2">
+      <c r="A53" s="2"/>
+      <c r="B53" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C53" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D53" s="8">
+        <v>46077.554594907408</v>
+      </c>
+      <c r="E53" s="8">
+        <v>46077.554594907408</v>
+      </c>
+      <c r="F53" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="G53" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="H53" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="I53" s="7">
+        <v>1422285</v>
+      </c>
+      <c r="J53" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="K53" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="L53" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="M53" s="10"/>
+      <c r="N53" s="10">
+        <v>3</v>
+      </c>
+      <c r="O53" s="7"/>
+    </row>
+    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A54" s="4"/>
+      <c r="B54" s="6"/>
+      <c r="C54" s="6"/>
+      <c r="D54" s="6"/>
+      <c r="E54" s="6"/>
+      <c r="F54" s="6"/>
+      <c r="G54" s="6"/>
+      <c r="H54" s="6"/>
+      <c r="I54" s="6"/>
+      <c r="J54" s="6"/>
+      <c r="K54" s="6"/>
+      <c r="L54" s="6"/>
+      <c r="M54" s="9">
         <v>0</v>
       </c>
-      <c r="N52" s="9">
-        <v>212</v>
-      </c>
-      <c r="O52" s="9">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="53" spans="1:15" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="3" t="s">
+      <c r="N54" s="9">
+        <v>227</v>
+      </c>
+      <c r="O54" s="9">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="55" spans="1:15" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B53" s="12" t="s">
+      <c r="B55" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C53" s="12"/>
-      <c r="D53" s="12"/>
-      <c r="E53" s="12"/>
-      <c r="F53" s="12"/>
-      <c r="G53" s="12"/>
-      <c r="H53" s="12"/>
-      <c r="I53" s="12"/>
-      <c r="J53" s="12"/>
-      <c r="K53" s="12"/>
-      <c r="L53" s="12"/>
-      <c r="M53" s="12"/>
-      <c r="N53" s="12"/>
-      <c r="O53" s="12"/>
-    </row>
-    <row r="54" spans="1:15" ht="21" x14ac:dyDescent="0.2">
-      <c r="A54" s="2"/>
-      <c r="B54" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C54" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D54" s="8">
-        <v>46027.666331018518</v>
-      </c>
-      <c r="E54" s="8">
-        <v>46027.666331018518</v>
-      </c>
-      <c r="F54" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="G54" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="H54" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="I54" s="7">
-        <v>1386388</v>
-      </c>
-      <c r="J54" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="K54" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="L54" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="M54" s="10"/>
-      <c r="N54" s="10">
-        <v>3</v>
-      </c>
-      <c r="O54" s="7"/>
-    </row>
-    <row r="55" spans="1:15" ht="21" x14ac:dyDescent="0.2">
-      <c r="A55" s="2"/>
-      <c r="B55" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C55" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D55" s="8">
-        <v>46027.694131944445</v>
-      </c>
-      <c r="E55" s="8">
-        <v>46027.694131944445</v>
-      </c>
-      <c r="F55" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="G55" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="H55" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="I55" s="7">
-        <v>1386388</v>
-      </c>
-      <c r="J55" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="K55" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="L55" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="M55" s="10"/>
-      <c r="N55" s="10">
-        <v>1</v>
-      </c>
-      <c r="O55" s="7"/>
+      <c r="C55" s="12"/>
+      <c r="D55" s="12"/>
+      <c r="E55" s="12"/>
+      <c r="F55" s="12"/>
+      <c r="G55" s="12"/>
+      <c r="H55" s="12"/>
+      <c r="I55" s="12"/>
+      <c r="J55" s="12"/>
+      <c r="K55" s="12"/>
+      <c r="L55" s="12"/>
+      <c r="M55" s="12"/>
+      <c r="N55" s="12"/>
+      <c r="O55" s="12"/>
     </row>
     <row r="56" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A56" s="2"/>
@@ -3125,38 +3128,38 @@
         <v>4</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="D56" s="8">
-        <v>46036.841574074075</v>
+        <v>46027.666331018518</v>
       </c>
       <c r="E56" s="8">
-        <v>46036.841574074075</v>
+        <v>46027.666331018518</v>
       </c>
       <c r="F56" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G56" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H56" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I56" s="7">
-        <v>1406206</v>
+        <v>1386388</v>
       </c>
       <c r="J56" s="5" t="s">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="K56" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L56" s="7" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="M56" s="10"/>
       <c r="N56" s="10">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="O56" s="7"/>
     </row>
@@ -3166,38 +3169,38 @@
         <v>4</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="D57" s="8">
-        <v>46059.905682870369</v>
+        <v>46027.694131944445</v>
       </c>
       <c r="E57" s="8">
-        <v>46059.905682870369</v>
+        <v>46027.694131944445</v>
       </c>
       <c r="F57" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G57" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H57" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I57" s="7">
-        <v>1411984</v>
+        <v>1386388</v>
       </c>
       <c r="J57" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K57" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L57" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="M57" s="10"/>
       <c r="N57" s="10">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="O57" s="7"/>
     </row>
@@ -3207,38 +3210,38 @@
         <v>4</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="D58" s="8">
-        <v>46064.60796296296</v>
+        <v>46036.841574074075</v>
       </c>
       <c r="E58" s="8">
-        <v>46064.60796296296</v>
+        <v>46036.841574074075</v>
       </c>
       <c r="F58" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G58" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H58" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I58" s="7">
-        <v>1411990</v>
+        <v>1406206</v>
       </c>
       <c r="J58" s="5" t="s">
-        <v>74</v>
+        <v>93</v>
       </c>
       <c r="K58" s="5" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="L58" s="7" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="M58" s="10"/>
       <c r="N58" s="10">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="O58" s="7"/>
     </row>
@@ -3251,35 +3254,35 @@
         <v>34</v>
       </c>
       <c r="D59" s="8">
-        <v>46065.655185185184</v>
+        <v>46059.905682870369</v>
       </c>
       <c r="E59" s="8">
-        <v>46065.655185185184</v>
+        <v>46059.905682870369</v>
       </c>
       <c r="F59" s="7" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="G59" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H59" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I59" s="7">
-        <v>1411990</v>
+        <v>1411984</v>
       </c>
       <c r="J59" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K59" s="5" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="L59" s="7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="M59" s="10"/>
       <c r="N59" s="10">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="O59" s="7"/>
     </row>
@@ -3289,38 +3292,38 @@
         <v>4</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="D60" s="8">
-        <v>46066.613657407404</v>
+        <v>46064.60796296296</v>
       </c>
       <c r="E60" s="8">
-        <v>46066.613657407404</v>
+        <v>46064.60796296296</v>
       </c>
       <c r="F60" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G60" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H60" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I60" s="7">
         <v>1411990</v>
       </c>
       <c r="J60" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K60" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L60" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="M60" s="10"/>
       <c r="N60" s="10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O60" s="7"/>
     </row>
@@ -3333,31 +3336,31 @@
         <v>35</v>
       </c>
       <c r="D61" s="8">
-        <v>46066.670127314814</v>
+        <v>46065.655185185184</v>
       </c>
       <c r="E61" s="8">
-        <v>46066.670127314814</v>
+        <v>46065.655185185184</v>
       </c>
       <c r="F61" s="7" t="s">
         <v>58</v>
       </c>
       <c r="G61" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H61" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I61" s="7">
         <v>1411990</v>
       </c>
       <c r="J61" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="K61" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L61" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="M61" s="10"/>
       <c r="N61" s="10">
@@ -3374,117 +3377,117 @@
         <v>36</v>
       </c>
       <c r="D62" s="8">
-        <v>46079.703912037039</v>
+        <v>46066.613657407404</v>
       </c>
       <c r="E62" s="8">
-        <v>46079.703912037039</v>
+        <v>46066.613657407404</v>
       </c>
       <c r="F62" s="7" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G62" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H62" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I62" s="7">
-        <v>1410767</v>
+        <v>1411990</v>
       </c>
       <c r="J62" s="5" t="s">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="K62" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L62" s="7" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="M62" s="10"/>
       <c r="N62" s="10">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="O62" s="7"/>
     </row>
     <row r="63" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A63" s="2"/>
       <c r="B63" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="D63" s="8">
-        <v>46028.907905092594</v>
+        <v>46066.670127314814</v>
       </c>
       <c r="E63" s="8">
-        <v>46028.907905092594</v>
+        <v>46066.670127314814</v>
       </c>
       <c r="F63" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G63" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H63" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I63" s="7">
-        <v>1394721</v>
+        <v>1411990</v>
       </c>
       <c r="J63" s="5" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="K63" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="L63" s="7" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="M63" s="10"/>
       <c r="N63" s="10">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="O63" s="7"/>
     </row>
     <row r="64" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A64" s="2"/>
       <c r="B64" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C64" s="7" t="s">
         <v>37</v>
       </c>
       <c r="D64" s="8">
-        <v>46029.6719212963</v>
+        <v>46079.703912037039</v>
       </c>
       <c r="E64" s="8">
-        <v>46029.6719212963</v>
+        <v>46079.703912037039</v>
       </c>
       <c r="F64" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G64" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H64" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I64" s="7">
-        <v>1394721</v>
+        <v>1410767</v>
       </c>
       <c r="J64" s="5" t="s">
-        <v>78</v>
+        <v>94</v>
       </c>
       <c r="K64" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="L64" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M64" s="10"/>
       <c r="N64" s="10">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O64" s="7"/>
     </row>
@@ -3494,38 +3497,38 @@
         <v>5</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="D65" s="8">
-        <v>46034.72855324074</v>
+        <v>46028.907905092594</v>
       </c>
       <c r="E65" s="8">
-        <v>46034.72855324074</v>
+        <v>46028.907905092594</v>
       </c>
       <c r="F65" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G65" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H65" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I65" s="7">
         <v>1394721</v>
       </c>
       <c r="J65" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K65" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L65" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M65" s="10"/>
       <c r="N65" s="10">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="O65" s="7"/>
     </row>
@@ -3535,38 +3538,38 @@
         <v>5</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D66" s="8">
-        <v>46037.838958333334</v>
+        <v>46029.6719212963</v>
       </c>
       <c r="E66" s="8">
-        <v>46037.838958333334</v>
+        <v>46029.6719212963</v>
       </c>
       <c r="F66" s="7" t="s">
         <v>59</v>
       </c>
       <c r="G66" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H66" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I66" s="7">
         <v>1394721</v>
       </c>
       <c r="J66" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K66" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L66" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M66" s="10"/>
       <c r="N66" s="10">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="O66" s="7"/>
     </row>
@@ -3576,38 +3579,38 @@
         <v>5</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D67" s="8">
-        <v>46042.727754629632</v>
+        <v>46034.72855324074</v>
       </c>
       <c r="E67" s="8">
-        <v>46042.727754629632</v>
+        <v>46034.72855324074</v>
       </c>
       <c r="F67" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G67" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H67" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I67" s="7">
         <v>1394721</v>
       </c>
       <c r="J67" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K67" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L67" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M67" s="10"/>
       <c r="N67" s="10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O67" s="7"/>
     </row>
@@ -3617,38 +3620,38 @@
         <v>5</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="D68" s="8">
-        <v>46043.627881944441</v>
+        <v>46037.838958333334</v>
       </c>
       <c r="E68" s="8">
-        <v>46043.627881944441</v>
+        <v>46037.838958333334</v>
       </c>
       <c r="F68" s="7" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G68" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H68" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I68" s="7">
-        <v>1410339</v>
+        <v>1394721</v>
       </c>
       <c r="J68" s="5" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="K68" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L68" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M68" s="10"/>
       <c r="N68" s="10">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="O68" s="7"/>
     </row>
@@ -3661,35 +3664,35 @@
         <v>41</v>
       </c>
       <c r="D69" s="8">
-        <v>46052.626018518517</v>
+        <v>46042.727754629632</v>
       </c>
       <c r="E69" s="8">
-        <v>46052.626018518517</v>
+        <v>46042.727754629632</v>
       </c>
       <c r="F69" s="7" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="G69" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H69" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I69" s="7">
-        <v>1411706</v>
+        <v>1394721</v>
       </c>
       <c r="J69" s="5" t="s">
         <v>79</v>
       </c>
       <c r="K69" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L69" s="7" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="M69" s="10"/>
       <c r="N69" s="10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O69" s="7"/>
     </row>
@@ -3699,38 +3702,38 @@
         <v>5</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="D70" s="8">
-        <v>46053.632291666669</v>
+        <v>46043.627881944441</v>
       </c>
       <c r="E70" s="8">
-        <v>46053.632291666669</v>
+        <v>46043.627881944441</v>
       </c>
       <c r="F70" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G70" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H70" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I70" s="7">
-        <v>1411708</v>
+        <v>1410339</v>
       </c>
       <c r="J70" s="5" t="s">
         <v>95</v>
       </c>
       <c r="K70" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L70" s="7" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="M70" s="10"/>
       <c r="N70" s="10">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="O70" s="7"/>
     </row>
@@ -3743,35 +3746,35 @@
         <v>42</v>
       </c>
       <c r="D71" s="8">
-        <v>46071.601446759261</v>
+        <v>46052.626018518517</v>
       </c>
       <c r="E71" s="8">
-        <v>46071.601446759261</v>
+        <v>46052.626018518517</v>
       </c>
       <c r="F71" s="7" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="G71" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H71" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I71" s="7">
-        <v>1418251</v>
+        <v>1411706</v>
       </c>
       <c r="J71" s="5" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="K71" s="5" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="L71" s="7" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="M71" s="10"/>
       <c r="N71" s="10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O71" s="7"/>
     </row>
@@ -3781,38 +3784,38 @@
         <v>5</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="D72" s="8">
-        <v>46076.679282407407</v>
+        <v>46053.632291666669</v>
       </c>
       <c r="E72" s="8">
-        <v>46076.679282407407</v>
+        <v>46053.632291666669</v>
       </c>
       <c r="F72" s="7" t="s">
         <v>58</v>
       </c>
       <c r="G72" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H72" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I72" s="7">
-        <v>1422511</v>
+        <v>1411708</v>
       </c>
       <c r="J72" s="5" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="K72" s="5" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="L72" s="7" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="M72" s="10"/>
       <c r="N72" s="10">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="O72" s="7"/>
     </row>
@@ -3822,38 +3825,38 @@
         <v>5</v>
       </c>
       <c r="C73" s="7" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="D73" s="8">
-        <v>46077.591944444444</v>
+        <v>46071.601446759261</v>
       </c>
       <c r="E73" s="8">
-        <v>46077.591944444444</v>
+        <v>46071.601446759261</v>
       </c>
       <c r="F73" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G73" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H73" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I73" s="7">
-        <v>1422511</v>
+        <v>1418251</v>
       </c>
       <c r="J73" s="5" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
       <c r="K73" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L73" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M73" s="10"/>
       <c r="N73" s="10">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O73" s="7"/>
     </row>
@@ -3863,120 +3866,120 @@
         <v>5</v>
       </c>
       <c r="C74" s="7" t="s">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="D74" s="8">
-        <v>46077.861296296294</v>
+        <v>46076.679282407407</v>
       </c>
       <c r="E74" s="8">
-        <v>46077.861296296294</v>
+        <v>46076.679282407407</v>
       </c>
       <c r="F74" s="7" t="s">
         <v>59</v>
       </c>
       <c r="G74" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H74" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I74" s="7">
         <v>1422511</v>
       </c>
       <c r="J74" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K74" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L74" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M74" s="10"/>
       <c r="N74" s="10">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="O74" s="7"/>
     </row>
     <row r="75" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A75" s="2"/>
       <c r="B75" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C75" s="7" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D75" s="8">
-        <v>46027.633611111109</v>
+        <v>46077.591944444444</v>
       </c>
       <c r="E75" s="8">
-        <v>46027.633611111109</v>
+        <v>46077.591944444444</v>
       </c>
       <c r="F75" s="7" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="G75" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H75" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I75" s="7">
-        <v>1404289</v>
+        <v>1422511</v>
       </c>
       <c r="J75" s="5" t="s">
         <v>83</v>
       </c>
       <c r="K75" s="5" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="L75" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M75" s="10"/>
       <c r="N75" s="10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O75" s="7"/>
     </row>
     <row r="76" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A76" s="2"/>
       <c r="B76" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C76" s="7" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="D76" s="8">
-        <v>46029.802372685182</v>
+        <v>46077.861296296294</v>
       </c>
       <c r="E76" s="8">
-        <v>46029.802372685182</v>
+        <v>46077.861296296294</v>
       </c>
       <c r="F76" s="7" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="G76" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H76" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I76" s="7">
-        <v>1394724</v>
+        <v>1422511</v>
       </c>
       <c r="J76" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K76" s="5" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="L76" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M76" s="10"/>
       <c r="N76" s="10">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="O76" s="7"/>
     </row>
@@ -3986,38 +3989,38 @@
         <v>6</v>
       </c>
       <c r="C77" s="7" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="D77" s="8">
-        <v>46030.908472222225</v>
+        <v>46027.633611111109</v>
       </c>
       <c r="E77" s="8">
-        <v>46030.908472222225</v>
+        <v>46027.633611111109</v>
       </c>
       <c r="F77" s="7" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G77" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H77" s="5" t="s">
         <v>70</v>
       </c>
       <c r="I77" s="7">
-        <v>1394724</v>
+        <v>1404289</v>
       </c>
       <c r="J77" s="5" t="s">
         <v>84</v>
       </c>
       <c r="K77" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L77" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M77" s="10"/>
       <c r="N77" s="10">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O77" s="7"/>
     </row>
@@ -4027,19 +4030,19 @@
         <v>6</v>
       </c>
       <c r="C78" s="7" t="s">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="D78" s="8">
-        <v>46031.590057870373</v>
+        <v>46029.802372685182</v>
       </c>
       <c r="E78" s="8">
-        <v>46031.590057870373</v>
+        <v>46029.802372685182</v>
       </c>
       <c r="F78" s="7" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G78" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H78" s="5" t="s">
         <v>70</v>
@@ -4048,17 +4051,17 @@
         <v>1394724</v>
       </c>
       <c r="J78" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K78" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L78" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M78" s="10"/>
       <c r="N78" s="10">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="O78" s="7"/>
     </row>
@@ -4068,38 +4071,38 @@
         <v>6</v>
       </c>
       <c r="C79" s="7" t="s">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="D79" s="8">
-        <v>46076.8827662037</v>
+        <v>46030.908472222225</v>
       </c>
       <c r="E79" s="8">
-        <v>46076.8827662037</v>
+        <v>46030.908472222225</v>
       </c>
       <c r="F79" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G79" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H79" s="5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I79" s="7">
-        <v>1422286</v>
+        <v>1394724</v>
       </c>
       <c r="J79" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="K79" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L79" s="7" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="M79" s="10"/>
       <c r="N79" s="10">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="O79" s="7"/>
     </row>
@@ -4109,34 +4112,34 @@
         <v>6</v>
       </c>
       <c r="C80" s="7" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D80" s="8">
-        <v>46078.867326388892</v>
+        <v>46031.590057870373</v>
       </c>
       <c r="E80" s="8">
-        <v>46078.867326388892</v>
+        <v>46031.590057870373</v>
       </c>
       <c r="F80" s="7" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G80" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H80" s="5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I80" s="7">
-        <v>1422286</v>
+        <v>1394724</v>
       </c>
       <c r="J80" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="K80" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L80" s="7" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="M80" s="10"/>
       <c r="N80" s="10">
@@ -4147,205 +4150,205 @@
     <row r="81" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A81" s="2"/>
       <c r="B81" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C81" s="7" t="s">
         <v>44</v>
       </c>
       <c r="D81" s="8">
-        <v>46024.795127314814</v>
+        <v>46076.8827662037</v>
       </c>
       <c r="E81" s="8">
-        <v>46024.795127314814</v>
+        <v>46076.8827662037</v>
       </c>
       <c r="F81" s="7" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G81" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H81" s="5" t="s">
         <v>70</v>
       </c>
       <c r="I81" s="7">
-        <v>1398335</v>
+        <v>1422286</v>
       </c>
       <c r="J81" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="K81" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L81" s="7" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="M81" s="10"/>
       <c r="N81" s="10">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="O81" s="7"/>
     </row>
     <row r="82" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A82" s="2"/>
       <c r="B82" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C82" s="7" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="D82" s="8">
-        <v>46024.795277777775</v>
+        <v>46078.867326388892</v>
       </c>
       <c r="E82" s="8">
-        <v>46024.795277777775</v>
+        <v>46078.867326388892</v>
       </c>
       <c r="F82" s="7" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="G82" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H82" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I82" s="7">
-        <v>1398335</v>
+        <v>1422286</v>
       </c>
       <c r="J82" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="K82" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L82" s="7" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="M82" s="10"/>
       <c r="N82" s="10">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O82" s="7"/>
     </row>
     <row r="83" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A83" s="2"/>
       <c r="B83" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C83" s="7" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="D83" s="8">
-        <v>46024.900324074071</v>
+        <v>46080.639293981483</v>
       </c>
       <c r="E83" s="8">
-        <v>46024.900324074071</v>
+        <v>46080.639293981483</v>
       </c>
       <c r="F83" s="7" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G83" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H83" s="5" t="s">
         <v>70</v>
       </c>
       <c r="I83" s="7">
-        <v>1398335</v>
+        <v>1422285</v>
       </c>
       <c r="J83" s="5" t="s">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="K83" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L83" s="7" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="M83" s="10"/>
       <c r="N83" s="10">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O83" s="7"/>
     </row>
     <row r="84" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A84" s="2"/>
       <c r="B84" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C84" s="7" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="D84" s="8">
-        <v>46028.866898148146</v>
+        <v>46080.716932870368</v>
       </c>
       <c r="E84" s="8">
-        <v>46028.866898148146</v>
+        <v>46080.716932870368</v>
       </c>
       <c r="F84" s="7" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="G84" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H84" s="5" t="s">
         <v>70</v>
       </c>
       <c r="I84" s="7">
-        <v>1402956</v>
+        <v>1422285</v>
       </c>
       <c r="J84" s="5" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="K84" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L84" s="7" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="M84" s="10"/>
       <c r="N84" s="10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O84" s="7"/>
     </row>
     <row r="85" spans="1:15" ht="21" x14ac:dyDescent="0.2">
       <c r="A85" s="2"/>
       <c r="B85" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C85" s="7" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="D85" s="8">
-        <v>46034.751261574071</v>
+        <v>46080.740543981483</v>
       </c>
       <c r="E85" s="8">
-        <v>46034.751261574071</v>
+        <v>46080.740543981483</v>
       </c>
       <c r="F85" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G85" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H85" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I85" s="7">
-        <v>1404958</v>
+        <v>1422285</v>
       </c>
       <c r="J85" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="K85" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L85" s="7" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="M85" s="10"/>
       <c r="N85" s="10">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="O85" s="7"/>
     </row>
@@ -4355,38 +4358,38 @@
         <v>7</v>
       </c>
       <c r="C86" s="7" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="D86" s="8">
-        <v>46062.904895833337</v>
+        <v>46024.795127314814</v>
       </c>
       <c r="E86" s="8">
-        <v>46062.904895833337</v>
+        <v>46024.795127314814</v>
       </c>
       <c r="F86" s="7" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="G86" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H86" s="5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I86" s="7">
-        <v>1412987</v>
+        <v>1398335</v>
       </c>
       <c r="J86" s="5" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="K86" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L86" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M86" s="10"/>
       <c r="N86" s="10">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="O86" s="7"/>
     </row>
@@ -4399,35 +4402,35 @@
         <v>45</v>
       </c>
       <c r="D87" s="8">
-        <v>46063.874467592592</v>
+        <v>46024.795277777775</v>
       </c>
       <c r="E87" s="8">
-        <v>46063.874467592592</v>
+        <v>46024.795277777775</v>
       </c>
       <c r="F87" s="7" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="G87" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H87" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I87" s="7">
-        <v>1412987</v>
+        <v>1398335</v>
       </c>
       <c r="J87" s="5" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="K87" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L87" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M87" s="10"/>
       <c r="N87" s="10">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O87" s="7"/>
     </row>
@@ -4437,38 +4440,38 @@
         <v>7</v>
       </c>
       <c r="C88" s="7" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="D88" s="8">
-        <v>46067.906875000001</v>
+        <v>46024.900324074071</v>
       </c>
       <c r="E88" s="8">
-        <v>46067.906875000001</v>
+        <v>46024.900324074071</v>
       </c>
       <c r="F88" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G88" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H88" s="5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I88" s="7">
-        <v>1411991</v>
+        <v>1398335</v>
       </c>
       <c r="J88" s="5" t="s">
         <v>98</v>
       </c>
       <c r="K88" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L88" s="7" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="M88" s="10"/>
       <c r="N88" s="10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O88" s="7"/>
     </row>
@@ -4478,38 +4481,38 @@
         <v>7</v>
       </c>
       <c r="C89" s="7" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="D89" s="8">
-        <v>46069.700543981482</v>
+        <v>46028.866898148146</v>
       </c>
       <c r="E89" s="8">
-        <v>46069.700543981482</v>
+        <v>46028.866898148146</v>
       </c>
       <c r="F89" s="7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G89" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H89" s="5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I89" s="7">
-        <v>1411991</v>
+        <v>1402956</v>
       </c>
       <c r="J89" s="5" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="K89" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L89" s="7" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="M89" s="10"/>
       <c r="N89" s="10">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="O89" s="7"/>
     </row>
@@ -4519,38 +4522,38 @@
         <v>7</v>
       </c>
       <c r="C90" s="7" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="D90" s="8">
-        <v>46077.65824074074</v>
+        <v>46034.751261574071</v>
       </c>
       <c r="E90" s="8">
-        <v>46077.65824074074</v>
+        <v>46034.751261574071</v>
       </c>
       <c r="F90" s="7" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="G90" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H90" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I90" s="7">
-        <v>1422285</v>
+        <v>1404958</v>
       </c>
       <c r="J90" s="5" t="s">
         <v>89</v>
       </c>
       <c r="K90" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L90" s="7" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="M90" s="10"/>
       <c r="N90" s="10">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="O90" s="7"/>
     </row>
@@ -4560,34 +4563,34 @@
         <v>7</v>
       </c>
       <c r="C91" s="7" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="D91" s="8">
-        <v>46078.881018518521</v>
+        <v>46062.904895833337</v>
       </c>
       <c r="E91" s="8">
-        <v>46078.881018518521</v>
+        <v>46062.904895833337</v>
       </c>
       <c r="F91" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G91" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H91" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I91" s="7">
-        <v>1423123</v>
+        <v>1412987</v>
       </c>
       <c r="J91" s="5" t="s">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="K91" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L91" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M91" s="10"/>
       <c r="N91" s="10">
@@ -4601,87 +4604,292 @@
         <v>7</v>
       </c>
       <c r="C92" s="7" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="D92" s="8">
-        <v>46079.901782407411</v>
+        <v>46063.874467592592</v>
       </c>
       <c r="E92" s="8">
-        <v>46079.901782407411</v>
+        <v>46063.874467592592</v>
       </c>
       <c r="F92" s="7" t="s">
         <v>60</v>
       </c>
       <c r="G92" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H92" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I92" s="7">
-        <v>1423123</v>
+        <v>1412987</v>
       </c>
       <c r="J92" s="5" t="s">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="K92" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L92" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M92" s="10"/>
       <c r="N92" s="10">
+        <v>5</v>
+      </c>
+      <c r="O92" s="7"/>
+    </row>
+    <row r="93" spans="1:15" ht="21" x14ac:dyDescent="0.2">
+      <c r="A93" s="2"/>
+      <c r="B93" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C93" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D93" s="8">
+        <v>46067.906875000001</v>
+      </c>
+      <c r="E93" s="8">
+        <v>46067.906875000001</v>
+      </c>
+      <c r="F93" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="G93" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="H93" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="I93" s="7">
+        <v>1411991</v>
+      </c>
+      <c r="J93" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="K93" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="L93" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="M93" s="10"/>
+      <c r="N93" s="10">
+        <v>3</v>
+      </c>
+      <c r="O93" s="7"/>
+    </row>
+    <row r="94" spans="1:15" ht="21" x14ac:dyDescent="0.2">
+      <c r="A94" s="2"/>
+      <c r="B94" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C94" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D94" s="8">
+        <v>46069.700543981482</v>
+      </c>
+      <c r="E94" s="8">
+        <v>46069.700543981482</v>
+      </c>
+      <c r="F94" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G94" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="H94" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="I94" s="7">
+        <v>1411991</v>
+      </c>
+      <c r="J94" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="K94" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="L94" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="M94" s="10"/>
+      <c r="N94" s="10">
+        <v>10</v>
+      </c>
+      <c r="O94" s="7"/>
+    </row>
+    <row r="95" spans="1:15" ht="21" x14ac:dyDescent="0.2">
+      <c r="A95" s="2"/>
+      <c r="B95" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C95" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D95" s="8">
+        <v>46077.65824074074</v>
+      </c>
+      <c r="E95" s="8">
+        <v>46077.65824074074</v>
+      </c>
+      <c r="F95" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="G95" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="H95" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="I95" s="7">
+        <v>1422285</v>
+      </c>
+      <c r="J95" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="K95" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="L95" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="M95" s="10"/>
+      <c r="N95" s="10">
         <v>1</v>
       </c>
-      <c r="O92" s="7"/>
-    </row>
-    <row r="93" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A93" s="4"/>
-      <c r="B93" s="6"/>
-      <c r="C93" s="6"/>
-      <c r="D93" s="6"/>
-      <c r="E93" s="6"/>
-      <c r="F93" s="6"/>
-      <c r="G93" s="6"/>
-      <c r="H93" s="6"/>
-      <c r="I93" s="6"/>
-      <c r="J93" s="6"/>
-      <c r="K93" s="6"/>
-      <c r="L93" s="6"/>
-      <c r="M93" s="9">
+      <c r="O95" s="7"/>
+    </row>
+    <row r="96" spans="1:15" ht="21" x14ac:dyDescent="0.2">
+      <c r="A96" s="2"/>
+      <c r="B96" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C96" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D96" s="8">
+        <v>46078.881018518521</v>
+      </c>
+      <c r="E96" s="8">
+        <v>46078.881018518521</v>
+      </c>
+      <c r="F96" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="G96" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="H96" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="I96" s="7">
+        <v>1423123</v>
+      </c>
+      <c r="J96" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="K96" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="L96" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="M96" s="10"/>
+      <c r="N96" s="10">
+        <v>1</v>
+      </c>
+      <c r="O96" s="7"/>
+    </row>
+    <row r="97" spans="1:15" ht="21" x14ac:dyDescent="0.2">
+      <c r="A97" s="2"/>
+      <c r="B97" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C97" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D97" s="8">
+        <v>46079.901782407411</v>
+      </c>
+      <c r="E97" s="8">
+        <v>46079.901782407411</v>
+      </c>
+      <c r="F97" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="G97" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="H97" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="I97" s="7">
+        <v>1423123</v>
+      </c>
+      <c r="J97" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="K97" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="L97" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="M97" s="10"/>
+      <c r="N97" s="10">
+        <v>1</v>
+      </c>
+      <c r="O97" s="7"/>
+    </row>
+    <row r="98" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A98" s="4"/>
+      <c r="B98" s="6"/>
+      <c r="C98" s="6"/>
+      <c r="D98" s="6"/>
+      <c r="E98" s="6"/>
+      <c r="F98" s="6"/>
+      <c r="G98" s="6"/>
+      <c r="H98" s="6"/>
+      <c r="I98" s="6"/>
+      <c r="J98" s="6"/>
+      <c r="K98" s="6"/>
+      <c r="L98" s="6"/>
+      <c r="M98" s="9">
         <v>0</v>
       </c>
-      <c r="N93" s="9">
-        <v>189</v>
-      </c>
-      <c r="O93" s="9">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="94" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A94" s="4"/>
-      <c r="B94" s="6"/>
-      <c r="C94" s="6"/>
-      <c r="D94" s="6"/>
-      <c r="E94" s="6"/>
-      <c r="F94" s="6"/>
-      <c r="G94" s="6"/>
-      <c r="H94" s="9">
-        <v>87</v>
-      </c>
-      <c r="I94" s="6"/>
-      <c r="J94" s="6"/>
-      <c r="K94" s="6"/>
-      <c r="L94" s="6"/>
-      <c r="M94" s="9">
+      <c r="N98" s="9">
+        <v>193</v>
+      </c>
+      <c r="O98" s="9">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="99" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A99" s="4"/>
+      <c r="B99" s="6"/>
+      <c r="C99" s="6"/>
+      <c r="D99" s="6"/>
+      <c r="E99" s="6"/>
+      <c r="F99" s="6"/>
+      <c r="G99" s="6"/>
+      <c r="H99" s="9">
+        <v>92</v>
+      </c>
+      <c r="I99" s="6"/>
+      <c r="J99" s="6"/>
+      <c r="K99" s="6"/>
+      <c r="L99" s="6"/>
+      <c r="M99" s="9">
         <v>0</v>
       </c>
-      <c r="N94" s="9">
-        <v>401</v>
-      </c>
-      <c r="O94" s="9">
-        <v>87</v>
+      <c r="N99" s="9">
+        <v>420</v>
+      </c>
+      <c r="O99" s="9">
+        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -4691,7 +4899,7 @@
     <mergeCell ref="M1:O1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="B3:O3"/>
-    <mergeCell ref="B53:O53"/>
+    <mergeCell ref="B55:O55"/>
   </mergeCells>
   <pageMargins left="0.78740157499999996" right="0.78740157499999996" top="0.984251969" bottom="0.984251969" header="0.4921259845" footer="0.4921259845"/>
 </worksheet>

</xml_diff>